<commit_message>
content(sheets): regenerate the spreadsheet template after the merge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -16361,12 +16361,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">records.title</t>
+          <t xml:space="preserve">records.search</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">سجلات المواطنين</t>
+          <t xml:space="preserve">بحث</t>
         </is>
       </c>
     </row>
@@ -16378,12 +16378,12 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">records.search</t>
+          <t xml:space="preserve">compare.match</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">بحث</t>
+          <t xml:space="preserve">تطابق</t>
         </is>
       </c>
     </row>
@@ -16395,12 +16395,12 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.match</t>
+          <t xml:space="preserve">compare.mismatch</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">تطابق</t>
+          <t xml:space="preserve">عدم تطابق</t>
         </is>
       </c>
     </row>
@@ -16412,12 +16412,12 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.mismatch</t>
+          <t xml:space="preserve">citation.title</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">عدم تطابق</t>
+          <t xml:space="preserve">إشعار انحراف زمني</t>
         </is>
       </c>
     </row>
@@ -16429,12 +16429,12 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation.title</t>
+          <t xml:space="preserve">citation.acknowledge</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">إشعار انحراف زمني</t>
+          <t xml:space="preserve">تم الاطلاع</t>
         </is>
       </c>
     </row>
@@ -16446,12 +16446,12 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation.acknowledge</t>
+          <t xml:space="preserve">window.settings</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">تم الاطلاع</t>
+          <t xml:space="preserve">الإعدادات</t>
         </is>
       </c>
     </row>
@@ -16463,12 +16463,12 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.directives</t>
+          <t xml:space="preserve">icon.internet</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">التوجيهات</t>
+          <t xml:space="preserve">الإنترنت</t>
         </is>
       </c>
     </row>
@@ -16480,12 +16480,12 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.scanner</t>
+          <t xml:space="preserve">icon.notes</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير الانحرافات</t>
+          <t xml:space="preserve">ملاحظات</t>
         </is>
       </c>
     </row>
@@ -16497,12 +16497,12 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.settings</t>
+          <t xml:space="preserve">icon.investigation</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الإعدادات</t>
+          <t xml:space="preserve">التحقيق</t>
         </is>
       </c>
     </row>
@@ -16514,12 +16514,12 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.directives</t>
+          <t xml:space="preserve">icon.mail</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">التوجيهات</t>
+          <t xml:space="preserve">البريد</t>
         </is>
       </c>
     </row>
@@ -16531,12 +16531,12 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.scanner</t>
+          <t xml:space="preserve">icon.account</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير الانحرافات</t>
+          <t xml:space="preserve">حساب المواطن</t>
         </is>
       </c>
     </row>
@@ -16548,12 +16548,12 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.records</t>
+          <t xml:space="preserve">icon.settings</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">السجلات</t>
+          <t xml:space="preserve">الإعدادات</t>
         </is>
       </c>
     </row>
@@ -16565,12 +16565,12 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.internet</t>
+          <t xml:space="preserve">tray.day</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الإنترنت</t>
+          <t xml:space="preserve">اليوم {0}</t>
         </is>
       </c>
     </row>
@@ -16582,12 +16582,12 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.lexicon</t>
+          <t xml:space="preserve">tray.stability</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">المعجم</t>
+          <t xml:space="preserve">الاستقرار: {0:0}%</t>
         </is>
       </c>
     </row>
@@ -16599,12 +16599,12 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.dialect</t>
+          <t xml:space="preserve">taskbar.desk</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اللهجات</t>
+          <t xml:space="preserve">العودة إلى المكتب</t>
         </is>
       </c>
     </row>
@@ -16616,12 +16616,12 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.material</t>
+          <t xml:space="preserve">briefing.title</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">المواد</t>
+          <t xml:space="preserve">اليوم {0} — الإحاطة الصباحية</t>
         </is>
       </c>
     </row>
@@ -16633,12 +16633,12 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.notes</t>
+          <t xml:space="preserve">results.title</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ملاحظات</t>
+          <t xml:space="preserve">اليوم {0} — تقرير المناوبة</t>
         </is>
       </c>
     </row>
@@ -16650,114 +16650,114 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.clueLog</t>
+          <t xml:space="preserve">briefing.newsHeader</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">سجل الأدلة</t>
+          <t xml:space="preserve">— أخبار الخط الزمني —</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ar</t>
+          <t xml:space="preserve">el</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tray.day</t>
+          <t xml:space="preserve">accept</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اليوم {0}</t>
+          <t xml:space="preserve">ΕΓΚΡΙΣΗ</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ar</t>
+          <t xml:space="preserve">el</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tray.stability</t>
+          <t xml:space="preserve">deny</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الاستقرار: {0:0}%</t>
+          <t xml:space="preserve">ΑΠΟΡΡΙΨΗ</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ar</t>
+          <t xml:space="preserve">el</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taskbar.desk</t>
+          <t xml:space="preserve">taskbar.start</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">العودة إلى المكتب</t>
+          <t xml:space="preserve">έναρξη</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ar</t>
+          <t xml:space="preserve">el</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.title</t>
+          <t xml:space="preserve">startmenu.settings</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اليوم {0} — الإحاطة الصباحية</t>
+          <t xml:space="preserve">Ρυθμίσεις</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ar</t>
+          <t xml:space="preserve">el</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.title</t>
+          <t xml:space="preserve">startmenu.screenOff</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اليوم {0} — تقرير المناوبة</t>
+          <t xml:space="preserve">Σβήσιμο οθόνης</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ar</t>
+          <t xml:space="preserve">el</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.newsHeader</t>
+          <t xml:space="preserve">startmenu.quit</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">— أخبار الخط الزمني —</t>
+          <t xml:space="preserve">Έξοδος από το παιχνίδι</t>
         </is>
       </c>
     </row>
@@ -16769,12 +16769,12 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">accept</t>
+          <t xml:space="preserve">briefing.masthead</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΕΓΚΡΙΣΗ</t>
+          <t xml:space="preserve">Η ΧΡΟΝΙΚΗ ΕΦΗΜΕΡΙΔΑ</t>
         </is>
       </c>
     </row>
@@ -16786,12 +16786,12 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">deny</t>
+          <t xml:space="preserve">briefing.start</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΑΠΟΡΡΙΨΗ</t>
+          <t xml:space="preserve">ΕΝΑΡΞΗ ΒΑΡΔΙΑΣ</t>
         </is>
       </c>
     </row>
@@ -16803,12 +16803,12 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taskbar.start</t>
+          <t xml:space="preserve">results.masthead</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">έναρξη</t>
+          <t xml:space="preserve">ΗΜΕΡΟΛΟΓΙΟ ΒΑΡΔΙΑΣ — ΑΠΟΓΕΥΜΑΤΙΝΗ ΕΚΔΟΣΗ</t>
         </is>
       </c>
     </row>
@@ -16820,12 +16820,12 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">startmenu.settings</t>
+          <t xml:space="preserve">results.goHome</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ρυθμίσεις</t>
+          <t xml:space="preserve">ΣΠΙΤΙ</t>
         </is>
       </c>
     </row>
@@ -16837,12 +16837,12 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">startmenu.screenOff</t>
+          <t xml:space="preserve">records.search</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σβήσιμο οθόνης</t>
+          <t xml:space="preserve">ΑΝΑΖΗΤΗΣΗ</t>
         </is>
       </c>
     </row>
@@ -16854,12 +16854,12 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">startmenu.quit</t>
+          <t xml:space="preserve">compare.match</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έξοδος από το παιχνίδι</t>
+          <t xml:space="preserve">ΤΑΙΡΙΑΖΕΙ</t>
         </is>
       </c>
     </row>
@@ -16871,12 +16871,12 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.masthead</t>
+          <t xml:space="preserve">compare.mismatch</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η ΧΡΟΝΙΚΗ ΕΦΗΜΕΡΙΔΑ</t>
+          <t xml:space="preserve">ΔΕΝ ΤΑΙΡΙΑΖΕΙ</t>
         </is>
       </c>
     </row>
@@ -16888,12 +16888,12 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.start</t>
+          <t xml:space="preserve">citation.title</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΕΝΑΡΞΗ ΒΑΡΔΙΑΣ</t>
+          <t xml:space="preserve">ΕΙΔΟΠΟΙΗΣΗ ΧΡΟΝΙΚΗΣ ΑΠΟΚΛΙΣΗΣ</t>
         </is>
       </c>
     </row>
@@ -16905,12 +16905,12 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.masthead</t>
+          <t xml:space="preserve">citation.acknowledge</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΗΜΕΡΟΛΟΓΙΟ ΒΑΡΔΙΑΣ — ΑΠΟΓΕΥΜΑΤΙΝΗ ΕΚΔΟΣΗ</t>
+          <t xml:space="preserve">Ελήφθη</t>
         </is>
       </c>
     </row>
@@ -16922,12 +16922,12 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.goHome</t>
+          <t xml:space="preserve">window.settings</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΣΠΙΤΙ</t>
+          <t xml:space="preserve">Ρυθμίσεις</t>
         </is>
       </c>
     </row>
@@ -16939,12 +16939,12 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">records.title</t>
+          <t xml:space="preserve">icon.internet</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Μητρώο Πολιτών</t>
+          <t xml:space="preserve">Διαδίκτυο</t>
         </is>
       </c>
     </row>
@@ -16956,12 +16956,12 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">records.search</t>
+          <t xml:space="preserve">icon.notes</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΑΝΑΖΗΤΗΣΗ</t>
+          <t xml:space="preserve">Σημειώσεις</t>
         </is>
       </c>
     </row>
@@ -16973,12 +16973,12 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.match</t>
+          <t xml:space="preserve">icon.investigation</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΤΑΙΡΙΑΖΕΙ</t>
+          <t xml:space="preserve">Έρευνα</t>
         </is>
       </c>
     </row>
@@ -16990,12 +16990,12 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.mismatch</t>
+          <t xml:space="preserve">icon.mail</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΔΕΝ ΤΑΙΡΙΑΖΕΙ</t>
+          <t xml:space="preserve">Αλληλογραφία</t>
         </is>
       </c>
     </row>
@@ -17007,12 +17007,12 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation.title</t>
+          <t xml:space="preserve">icon.account</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΕΙΔΟΠΟΙΗΣΗ ΧΡΟΝΙΚΗΣ ΑΠΟΚΛΙΣΗΣ</t>
+          <t xml:space="preserve">Λογαριασμός πολίτη</t>
         </is>
       </c>
     </row>
@@ -17024,12 +17024,12 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation.acknowledge</t>
+          <t xml:space="preserve">icon.settings</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ελήφθη</t>
+          <t xml:space="preserve">Ρυθμίσεις</t>
         </is>
       </c>
     </row>
@@ -17041,12 +17041,12 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.directives</t>
+          <t xml:space="preserve">tray.day</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Οδηγίες</t>
+          <t xml:space="preserve">Ημέρα {0}</t>
         </is>
       </c>
     </row>
@@ -17058,12 +17058,12 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.scanner</t>
+          <t xml:space="preserve">tray.stability</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναφορά αποκλίσεων</t>
+          <t xml:space="preserve">Σταθερότητα: {0:0}%</t>
         </is>
       </c>
     </row>
@@ -17075,12 +17075,12 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.settings</t>
+          <t xml:space="preserve">taskbar.desk</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ρυθμίσεις</t>
+          <t xml:space="preserve">&lt; Γραφείο</t>
         </is>
       </c>
     </row>
@@ -17092,12 +17092,12 @@
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.directives</t>
+          <t xml:space="preserve">briefing.title</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Οδηγίες</t>
+          <t xml:space="preserve">Ημέρα {0} — Πρωινή ενημέρωση</t>
         </is>
       </c>
     </row>
@@ -17109,12 +17109,12 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.scanner</t>
+          <t xml:space="preserve">results.title</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναφορά αποκλίσεων</t>
+          <t xml:space="preserve">Ημέρα {0} — Αναφορά βάρδιας</t>
         </is>
       </c>
     </row>
@@ -17126,214 +17126,10 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.records</t>
+          <t xml:space="preserve">briefing.newsHeader</t>
         </is>
       </c>
       <c r="C57" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Μητρώο</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B58" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">icon.internet</t>
-        </is>
-      </c>
-      <c r="C58" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Διαδίκτυο</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B59" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">icon.lexicon</t>
-        </is>
-      </c>
-      <c r="C59" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Λεξικό</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B60" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">icon.dialect</t>
-        </is>
-      </c>
-      <c r="C60" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Διάλεκτος</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">icon.material</t>
-        </is>
-      </c>
-      <c r="C61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Υλικά</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">icon.notes</t>
-        </is>
-      </c>
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Σημειώσεις</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">icon.clueLog</t>
-        </is>
-      </c>
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ενδείξεις</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B64" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tray.day</t>
-        </is>
-      </c>
-      <c r="C64" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ημέρα {0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B65" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tray.stability</t>
-        </is>
-      </c>
-      <c r="C65" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Σταθερότητα: {0:0}%</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B66" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">taskbar.desk</t>
-        </is>
-      </c>
-      <c r="C66" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt; Γραφείο</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B67" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">briefing.title</t>
-        </is>
-      </c>
-      <c r="C67" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ημέρα {0} — Πρωινή ενημέρωση</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B68" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">results.title</t>
-        </is>
-      </c>
-      <c r="C68" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ημέρα {0} — Αναφορά βάρδιας</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">el</t>
-        </is>
-      </c>
-      <c r="B69" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">briefing.newsHeader</t>
-        </is>
-      </c>
-      <c r="C69" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">— ΕΙΔΗΣΕΙΣ ΧΡΟΝΟΓΡΑΜΜΗΣ —</t>
         </is>

</xml_diff>

<commit_message>
build(data): Generate World with the displaced on day 5, the famous on day 6, and the sheet template
The day plans, the two new rule assets (Rule_DisplacedReturns, Rule_ReturnHome),
the Future era named "2150", the translation notice on night 3 and the home
questions from day 5, as Generate World writes them; the content spreadsheet
template rewritten on the map (the days' lies note names FakeDisplaced).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -4498,7 +4498,7 @@
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the lies enabled this day (FalseOrigin, PoorPosingAsRich, DoctoredIdentity); a traveller draws among those that fit their kind</t>
+          <t xml:space="preserve">the lies enabled this day (FalseOrigin, PoorPosingAsRich, DoctoredIdentity, FakeDisplaced); a traveller draws among those that fit their kind</t>
         </is>
       </c>
     </row>
@@ -14711,10 +14711,10 @@
     <col min="3" max="3" width="8" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="15" style="1" customWidth="1"/>
-    <col min="6" max="6" width="47" style="1" customWidth="1"/>
+    <col min="6" max="6" width="35" style="1" customWidth="1"/>
     <col min="7" max="7" width="39" style="1" customWidth="1"/>
     <col min="8" max="8" width="46" style="1" customWidth="1"/>
-    <col min="9" max="9" width="32" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10" style="1" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
@@ -14798,7 +14798,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PoorPosingAsRich|DoctoredIdentity|FalseOrigin</t>
+          <t xml:space="preserve">PoorPosingAsRich|DoctoredIdentity</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
@@ -14812,7 +14812,7 @@
         </is>
       </c>
       <c r="J2">
-        <v>0.05</v>
+        <v>0.0</v>
       </c>
       <c r="K2">
         <v>0.0</v>
@@ -14840,7 +14840,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">FalseOrigin</t>
+          <t xml:space="preserve">PoorPosingAsRich|DoctoredIdentity</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
@@ -14853,13 +14853,8 @@
           <t xml:space="preserve">Rule_NoAncientEgypt|Rule_DressForDestination</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">aspasia|banzhao|arib|khwarizmi</t>
-        </is>
-      </c>
       <c r="J3">
-        <v>0.05</v>
+        <v>0.0</v>
       </c>
       <c r="K3">
         <v>0.1</v>
@@ -14913,31 +14908,16 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displaced</t>
+          <t xml:space="preserve">RichTourist</t>
         </is>
       </c>
       <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Displaced</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -15025,7 +15005,7 @@
   <cols>
     <col min="1" max="1" width="8" style="1" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9" style="1" customWidth="1"/>
     <col min="4" max="4" width="11" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -15048,36 +15028,6 @@
       <c r="D1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">blueprint</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">senenmut</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">socrates</t>
         </is>
       </c>
     </row>
@@ -19737,11 +19687,11 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Budget cuts close the interpreter pool. From today, foreign speech reaches the desk untranslated but for its key words; translators are sold at Home. Papers are still filled in English.</t>
+          <t xml:space="preserve">Budget cuts close the interpreter pool. From tomorrow, the displaced reach the desk speaking their own tongues, untranslated but for their key words; Speech translators are sold at Home tonight. Papers are still filled in English.</t>
         </is>
       </c>
       <c r="C2">

</xml_diff>

<commit_message>
content(generated): Generate World with the stability strings taking the formatted value; the sheet template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -20013,7 +20013,7 @@
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الاستقرار: {0:0}%</t>
+          <t xml:space="preserve">الاستقرار: {0}</t>
         </is>
       </c>
     </row>
@@ -20489,7 +20489,7 @@
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σταθερότητα: {0:0}%</t>
+          <t xml:space="preserve">Σταθερότητα: {0}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(news): the paper's Debt Relief count reads for any count; phase 9's as-built notes
"Citizens who left on Debt Relief yesterday: 1." replaces "1 citizens
left..." (the feature play showed the singular). The plan's phase 9 notes
are rewritten for the merged branch: the one rule path (what was folded
and dropped at the phase 11 merge), the renumbered enums, L3, L10 and L4's
poor variant with their decisions, the phase 23 changes and the K5 fix.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -18157,7 +18157,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="60" style="1" customWidth="1"/>
-    <col min="2" max="2" width="49" style="1" customWidth="1"/>
+    <col min="2" max="2" width="54" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">{count} citizens left on Debt Relief yesterday.</t>
+          <t xml:space="preserve">Citizens who left on Debt Relief yesterday: {count}.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(generated): Generate World with the tuned day chances; the sheet template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -16014,10 +16014,10 @@
         <v>0.0</v>
       </c>
       <c r="K3">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="L3">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content(steps): the default set's facts and dress keep the kinds' first days
The steps checklist shows the default set until the arrival paper is read
(the personalities spec's B5); its place facts now start on day 4 and its
dress on day 2, as every kind's set does, so reading the arrival paper only
adds steps (on day 1 the facts and dress rows no longer show, then vanish).
FEATURES 48 regains the B5 sentence the main 6d0c5d0 merge's resolution
dropped. Generate World rewrites the library's steps and the template.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -18473,6 +18473,9 @@
           <t xml:space="preserve">FirstUncheckedField</t>
         </is>
       </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -18558,6 +18561,9 @@
         <is>
           <t xml:space="preserve">CostumeClaimed</t>
         </is>
+      </c>
+      <c r="K9">
+        <v>2</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
build(data): the sheet template on main 164a15b's tuned days
Write Content Spreadsheet Template after Generate World on the merge
(Generate World 0 errors, the validator clean; no generated asset's
content changed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -15975,10 +15975,10 @@
         <v>0.0</v>
       </c>
       <c r="K3">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="L3">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content(orders): Generate World and the template with the Orders content
Generate World (0 errors, 0 warnings; a second run changed nothing) and
the validator (no issues): the Orders strings in the eight string tables
(icon.orders in every culture), the translators as Interview nodes after
Interview Protocols, and the translation notice on night 2 (day 3's
paper) in its new words. Write Content Spreadsheet Template adds the
packs' requires column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -14101,17 +14101,32 @@
     <row r="574">
       <c r="A574" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tongues</t>
+          <t xml:space="preserve">packs</t>
+        </is>
+      </c>
+      <c r="B574" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requires</t>
         </is>
       </c>
       <c r="C574" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
+          <t xml:space="preserve">text list</t>
+        </is>
+      </c>
+      <c r="D574" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no items (left out of the JSON)</t>
         </is>
       </c>
       <c r="E574" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">one row per item of the list $.translation.tongues, in order; a row's name is id, unique</t>
+          <t xml:space="preserve">separate items with |</t>
+        </is>
+      </c>
+      <c r="F574" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the upgrade ids the translator's Orders node needs owned first (interview_protocols); blank: none</t>
         </is>
       </c>
     </row>
@@ -14121,24 +14136,14 @@
           <t xml:space="preserve">tongues</t>
         </is>
       </c>
-      <c r="B575" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
       <c r="C575" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D575" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">Rows</t>
         </is>
       </c>
       <c r="E575" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">part of the row's name</t>
+          <t xml:space="preserve">one row per item of the list $.translation.tongues, in order; a row's name is id, unique</t>
         </is>
       </c>
     </row>
@@ -14150,7 +14155,7 @@
       </c>
       <c r="B576" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">displayName</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="C576" s="1" t="inlineStr">
@@ -14160,7 +14165,12 @@
       </c>
       <c r="D576" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E576" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
         </is>
       </c>
     </row>
@@ -14172,7 +14182,7 @@
       </c>
       <c r="B577" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">script</t>
+          <t xml:space="preserve">displayName</t>
         </is>
       </c>
       <c r="C577" s="1" t="inlineStr">
@@ -14183,11 +14193,6 @@
       <c r="D577" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">empty text</t>
-        </is>
-      </c>
-      <c r="E577" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">names a row of 'scripts'</t>
         </is>
       </c>
     </row>
@@ -14199,7 +14204,7 @@
       </c>
       <c r="B578" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">pack</t>
+          <t xml:space="preserve">script</t>
         </is>
       </c>
       <c r="C578" s="1" t="inlineStr">
@@ -14214,7 +14219,7 @@
       </c>
       <c r="E578" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">names a row of 'packs'</t>
+          <t xml:space="preserve">names a row of 'scripts'</t>
         </is>
       </c>
     </row>
@@ -14226,15 +14231,42 @@
       </c>
       <c r="B579" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">pack</t>
+        </is>
+      </c>
+      <c r="C579" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D579" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E579" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'packs'</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tongues</t>
+        </is>
+      </c>
+      <c r="B580" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">glyphs</t>
         </is>
       </c>
-      <c r="C579" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D579" s="1" t="inlineStr">
+      <c r="C580" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D580" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">empty text</t>
         </is>
@@ -23347,12 +23379,12 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.investigation</t>
+          <t xml:space="preserve">icon.orders</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">التحقيق</t>
+          <t xml:space="preserve">الطلبات</t>
         </is>
       </c>
     </row>
@@ -23364,12 +23396,12 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.mail</t>
+          <t xml:space="preserve">icon.investigation</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">البريد</t>
+          <t xml:space="preserve">التحقيق</t>
         </is>
       </c>
     </row>
@@ -23381,12 +23413,12 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.account</t>
+          <t xml:space="preserve">icon.mail</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">حساب المواطن</t>
+          <t xml:space="preserve">البريد</t>
         </is>
       </c>
     </row>
@@ -23398,12 +23430,12 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.settings</t>
+          <t xml:space="preserve">icon.account</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الإعدادات</t>
+          <t xml:space="preserve">حساب المواطن</t>
         </is>
       </c>
     </row>
@@ -23415,12 +23447,12 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tray.day</t>
+          <t xml:space="preserve">icon.settings</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اليوم {0}</t>
+          <t xml:space="preserve">الإعدادات</t>
         </is>
       </c>
     </row>
@@ -23432,12 +23464,12 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tray.stability</t>
+          <t xml:space="preserve">tray.day</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الاستقرار: {0}</t>
+          <t xml:space="preserve">اليوم {0}</t>
         </is>
       </c>
     </row>
@@ -23449,12 +23481,12 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taskbar.desk</t>
+          <t xml:space="preserve">tray.stability</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">العودة إلى المكتب</t>
+          <t xml:space="preserve">الاستقرار: {0}</t>
         </is>
       </c>
     </row>
@@ -23466,12 +23498,12 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.title</t>
+          <t xml:space="preserve">taskbar.desk</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اليوم {0} — الإحاطة الصباحية</t>
+          <t xml:space="preserve">العودة إلى المكتب</t>
         </is>
       </c>
     </row>
@@ -23483,12 +23515,12 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.title</t>
+          <t xml:space="preserve">briefing.title</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">اليوم {0} — تقرير المناوبة</t>
+          <t xml:space="preserve">اليوم {0} — الإحاطة الصباحية</t>
         </is>
       </c>
     </row>
@@ -23500,29 +23532,29 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.newsHeader</t>
+          <t xml:space="preserve">results.title</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">— أخبار الخط الزمني —</t>
+          <t xml:space="preserve">اليوم {0} — تقرير المناوبة</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">el</t>
+          <t xml:space="preserve">ar</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">accept</t>
+          <t xml:space="preserve">briefing.newsHeader</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΕΓΚΡΙΣΗ</t>
+          <t xml:space="preserve">— أخبار الخط الزمني —</t>
         </is>
       </c>
     </row>
@@ -23534,12 +23566,12 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">deny</t>
+          <t xml:space="preserve">accept</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΑΠΟΡΡΙΨΗ</t>
+          <t xml:space="preserve">ΕΓΚΡΙΣΗ</t>
         </is>
       </c>
     </row>
@@ -23551,12 +23583,12 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taskbar.start</t>
+          <t xml:space="preserve">deny</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">έναρξη</t>
+          <t xml:space="preserve">ΑΠΟΡΡΙΨΗ</t>
         </is>
       </c>
     </row>
@@ -23568,12 +23600,12 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">startmenu.settings</t>
+          <t xml:space="preserve">taskbar.start</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ρυθμίσεις</t>
+          <t xml:space="preserve">έναρξη</t>
         </is>
       </c>
     </row>
@@ -23585,12 +23617,12 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">startmenu.screenOff</t>
+          <t xml:space="preserve">startmenu.settings</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σβήσιμο οθόνης</t>
+          <t xml:space="preserve">Ρυθμίσεις</t>
         </is>
       </c>
     </row>
@@ -23602,12 +23634,12 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">startmenu.quit</t>
+          <t xml:space="preserve">startmenu.screenOff</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έξοδος από το παιχνίδι</t>
+          <t xml:space="preserve">Σβήσιμο οθόνης</t>
         </is>
       </c>
     </row>
@@ -23619,12 +23651,12 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.masthead</t>
+          <t xml:space="preserve">startmenu.quit</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η ΧΡΟΝΙΚΗ ΕΦΗΜΕΡΙΔΑ</t>
+          <t xml:space="preserve">Έξοδος από το παιχνίδι</t>
         </is>
       </c>
     </row>
@@ -23636,12 +23668,12 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.start</t>
+          <t xml:space="preserve">briefing.masthead</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΕΝΑΡΞΗ ΒΑΡΔΙΑΣ</t>
+          <t xml:space="preserve">Η ΧΡΟΝΙΚΗ ΕΦΗΜΕΡΙΔΑ</t>
         </is>
       </c>
     </row>
@@ -23653,12 +23685,12 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.masthead</t>
+          <t xml:space="preserve">briefing.start</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΗΜΕΡΟΛΟΓΙΟ ΒΑΡΔΙΑΣ — ΑΠΟΓΕΥΜΑΤΙΝΗ ΕΚΔΟΣΗ</t>
+          <t xml:space="preserve">ΕΝΑΡΞΗ ΒΑΡΔΙΑΣ</t>
         </is>
       </c>
     </row>
@@ -23670,12 +23702,12 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.goHome</t>
+          <t xml:space="preserve">results.masthead</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΣΠΙΤΙ</t>
+          <t xml:space="preserve">ΗΜΕΡΟΛΟΓΙΟ ΒΑΡΔΙΑΣ — ΑΠΟΓΕΥΜΑΤΙΝΗ ΕΚΔΟΣΗ</t>
         </is>
       </c>
     </row>
@@ -23687,12 +23719,12 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">records.search</t>
+          <t xml:space="preserve">results.goHome</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΑΝΑΖΗΤΗΣΗ</t>
+          <t xml:space="preserve">ΣΠΙΤΙ</t>
         </is>
       </c>
     </row>
@@ -23704,12 +23736,12 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.match</t>
+          <t xml:space="preserve">records.search</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΤΑΙΡΙΑΖΕΙ</t>
+          <t xml:space="preserve">ΑΝΑΖΗΤΗΣΗ</t>
         </is>
       </c>
     </row>
@@ -23721,12 +23753,12 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">compare.mismatch</t>
+          <t xml:space="preserve">compare.match</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΔΕΝ ΤΑΙΡΙΑΖΕΙ</t>
+          <t xml:space="preserve">ΤΑΙΡΙΑΖΕΙ</t>
         </is>
       </c>
     </row>
@@ -23738,12 +23770,12 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation.title</t>
+          <t xml:space="preserve">compare.mismatch</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ΕΙΔΟΠΟΙΗΣΗ ΧΡΟΝΙΚΗΣ ΑΠΟΚΛΙΣΗΣ</t>
+          <t xml:space="preserve">ΔΕΝ ΤΑΙΡΙΑΖΕΙ</t>
         </is>
       </c>
     </row>
@@ -23755,12 +23787,12 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation.acknowledge</t>
+          <t xml:space="preserve">citation.title</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ελήφθη</t>
+          <t xml:space="preserve">ΕΙΔΟΠΟΙΗΣΗ ΧΡΟΝΙΚΗΣ ΑΠΟΚΛΙΣΗΣ</t>
         </is>
       </c>
     </row>
@@ -23772,12 +23804,12 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">window.settings</t>
+          <t xml:space="preserve">citation.acknowledge</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ρυθμίσεις</t>
+          <t xml:space="preserve">Ελήφθη</t>
         </is>
       </c>
     </row>
@@ -23789,12 +23821,12 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.internet</t>
+          <t xml:space="preserve">window.settings</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Διαδίκτυο</t>
+          <t xml:space="preserve">Ρυθμίσεις</t>
         </is>
       </c>
     </row>
@@ -23806,12 +23838,12 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.notes</t>
+          <t xml:space="preserve">icon.internet</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σημειώσεις</t>
+          <t xml:space="preserve">Διαδίκτυο</t>
         </is>
       </c>
     </row>
@@ -23823,12 +23855,12 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.investigation</t>
+          <t xml:space="preserve">icon.notes</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έρευνα</t>
+          <t xml:space="preserve">Σημειώσεις</t>
         </is>
       </c>
     </row>
@@ -23840,12 +23872,12 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.mail</t>
+          <t xml:space="preserve">icon.orders</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αλληλογραφία</t>
+          <t xml:space="preserve">Παραγγελίες</t>
         </is>
       </c>
     </row>
@@ -23857,12 +23889,12 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.account</t>
+          <t xml:space="preserve">icon.investigation</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λογαριασμός πολίτη</t>
+          <t xml:space="preserve">Έρευνα</t>
         </is>
       </c>
     </row>
@@ -23874,12 +23906,12 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">icon.settings</t>
+          <t xml:space="preserve">icon.mail</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ρυθμίσεις</t>
+          <t xml:space="preserve">Αλληλογραφία</t>
         </is>
       </c>
     </row>
@@ -23891,12 +23923,12 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tray.day</t>
+          <t xml:space="preserve">icon.account</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ημέρα {0}</t>
+          <t xml:space="preserve">Λογαριασμός πολίτη</t>
         </is>
       </c>
     </row>
@@ -23908,12 +23940,12 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tray.stability</t>
+          <t xml:space="preserve">icon.settings</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σταθερότητα: {0}</t>
+          <t xml:space="preserve">Ρυθμίσεις</t>
         </is>
       </c>
     </row>
@@ -23925,12 +23957,12 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taskbar.desk</t>
+          <t xml:space="preserve">tray.day</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt; Γραφείο</t>
+          <t xml:space="preserve">Ημέρα {0}</t>
         </is>
       </c>
     </row>
@@ -23942,12 +23974,12 @@
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">briefing.title</t>
+          <t xml:space="preserve">tray.stability</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ημέρα {0} — Πρωινή ενημέρωση</t>
+          <t xml:space="preserve">Σταθερότητα: {0}</t>
         </is>
       </c>
     </row>
@@ -23959,12 +23991,12 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">results.title</t>
+          <t xml:space="preserve">taskbar.desk</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ημέρα {0} — Αναφορά βάρδιας</t>
+          <t xml:space="preserve">&lt; Γραφείο</t>
         </is>
       </c>
     </row>
@@ -23976,10 +24008,44 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">briefing.title</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ημέρα {0} — Πρωινή ενημέρωση</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">el</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">results.title</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ημέρα {0} — Αναφορά βάρδιας</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">el</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">briefing.newsHeader</t>
         </is>
       </c>
-      <c r="C57" s="1" t="inlineStr">
+      <c r="C59" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">— ΕΙΔΗΣΕΙΣ ΧΡΟΝΟΓΡΑΜΜΗΣ —</t>
         </is>
@@ -24063,7 +24129,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Budget cuts close the interpreter pool. From tomorrow, the displaced reach the desk speaking their own tongues, untranslated but for their key words; Speech translators are sold at Home tonight. Papers are still filled in English.</t>
+          <t xml:space="preserve">Budget cuts close the interpreter pool. From the day after tomorrow, the displaced reach the desk speaking their own tongues, untranslated but for their key words. Order Interview Protocols today and a Speech translator tomorrow in Orders: each arrives the morning after it is ordered. Papers are still filled in English.</t>
         </is>
       </c>
       <c r="C2">
@@ -24194,6 +24260,7 @@
     <col min="1" max="1" width="15" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="21" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -24212,6 +24279,11 @@
           <t xml:space="preserve">spokenCost</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requires</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -24227,6 +24299,11 @@
       <c r="C2">
         <v>80</v>
       </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">interview_protocols</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -24241,6 +24318,11 @@
       </c>
       <c r="C3">
         <v>80</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">interview_protocols</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
build(data,scene): Generate World with the House tree; the House panel built
Generate World on main 23165bd plus this branch: the 18 house upgrades
and their effects in Assets/Data/World/Home, listed in ContentLibrary_Main
with the radio block (a second and third run change nothing; cases.txt is
byte-identical before and after). Build Home UI: the expenses panel at
900 x 780, the House panel at 1720 x 900 with its tree area, detail strip
and Buy, the old rows container gone (rebuilt identically twice).
OfficeGameplay and TitleScene rebuild identically by semantic dump and
stay as committed. The content spreadsheet template carries the home
sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -103,6 +103,9 @@
     <sheet name="scriptFonts" sheetId="99" r:id="rId99"/>
     <sheet name="packs" sheetId="100" r:id="rId100"/>
     <sheet name="tongues" sheetId="101" r:id="rId101"/>
+    <sheet name="home" sheetId="102" r:id="rId102"/>
+    <sheet name="homeRadio" sheetId="103" r:id="rId103"/>
+    <sheet name="homeUpgrades" sheetId="104" r:id="rId104"/>
   </sheets>
 </workbook>
 </file>
@@ -15138,6 +15141,509 @@
         </is>
       </c>
     </row>
+    <row r="612">
+      <c r="A612" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">home</t>
+        </is>
+      </c>
+      <c r="C612" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single</t>
+        </is>
+      </c>
+      <c r="E612" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row: the object $.home</t>
+        </is>
+      </c>
+      <c r="F612" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home's house upgrades and the radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">home</t>
+        </is>
+      </c>
+      <c r="B613" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">radioUpgrade</t>
+        </is>
+      </c>
+      <c r="C613" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D613" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F613" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the house upgrade whose ownership plays a radio line on the sleep panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeRadio</t>
+        </is>
+      </c>
+      <c r="C614" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E614" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.radio, in order</t>
+        </is>
+      </c>
+      <c r="F614" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the radio's lines: one a night, in order by the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeRadio</t>
+        </is>
+      </c>
+      <c r="B615" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C615" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D615" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="C616" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E616" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.upgrades, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+      <c r="F616" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the House tree: every effect never takes a knob below 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B617" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C617" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D617" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E617" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F617" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the upgrade's id (saved as owned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B618" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C618" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D618" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B619" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">category</t>
+        </is>
+      </c>
+      <c r="C619" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D619" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E619" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: Food, Housing, Security, Health, Comfort</t>
+        </is>
+      </c>
+      <c r="F619" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its column in the House panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B620" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cost</t>
+        </is>
+      </c>
+      <c r="C620" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D620" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F620" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the one-off price in cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B621" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">upkeep</t>
+        </is>
+      </c>
+      <c r="C621" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D621" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F621" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr a night the household pays once it is owned (0: none)</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B622" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requires</t>
+        </is>
+      </c>
+      <c r="C622" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text list</t>
+        </is>
+      </c>
+      <c r="D622" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no items</t>
+        </is>
+      </c>
+      <c r="E622" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">separate items with |</t>
+        </is>
+      </c>
+      <c r="F622" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the house upgrades it needs owned first (ids of this sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">householdExpense</t>
+        </is>
+      </c>
+      <c r="C623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr a night on rent and utilities (negative saves)</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sicknessChance</t>
+        </is>
+      </c>
+      <c r="C624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added to each member's nightly chance to worsen (-0.05 = 5 points less)</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">careCost</t>
+        </is>
+      </c>
+      <c r="C625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr on each treatment (negative cheaper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medicalDrain</t>
+        </is>
+      </c>
+      <c r="C626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr on each condition point's nightly drain (negative lowers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood</t>
+        </is>
+      </c>
+      <c r="C627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the household's mood points (a sick member's nightly recovery chance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInChance</t>
+        </is>
+      </c>
+      <c r="C628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added to the nightly break-in chance (-0.03 = 3 points less)</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInShare</t>
+        </is>
+      </c>
+      <c r="C629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added to the share of the wallet a break-in takes</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
+      <c r="C630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the House panel's line under its name</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -15329,6 +15835,262 @@
       <c r="E3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">𓄿𓃀𓍿𓂧𓇋𓆑𓎼𓉔𓇌𓆓𓎡𓃭𓅓𓈖𓂝𓊪𓈎𓂋𓋴𓏏𓅱𓎛𓏲𓐍𓏭𓊃</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet102.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">radioUpgrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_radio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet103.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tonight's weather: overcast, with a chance of interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Directorate reminds listeners that sleep is a privilege of the solvent.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet104.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="17" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="8" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">category</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cost</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">upkeep</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requires</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">householdExpense</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sicknessChance</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">careCost</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medicalDrain</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInChance</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInShare</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_rations_b</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ration Card, Tier B</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Food</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>40</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>-0.02</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tier B paste comes in two colours. The kid prefers the green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_veg_box</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vegetable Box</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Food</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>90</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_rations_b</t>
+        </is>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>-0.04</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Real vegetables, by drone, once a week. The carrots are small, but they are carrots.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
build(data,scene): the shorter house names generated; the House rebuilt at 720p's scale
Generate World writes the eight renamed house upgrades and their effects
(a second run changes nothing; cases.txt is byte-identical). Build Home
UI: the canvas scales from 1920 x 1080, the House panel is 1840 x 920
lowered 30 px, the detail strip at 24 px (rebuilt identically twice).
OfficeGameplay and TitleScene rebuild identically and stay as committed.
The content template carries the new names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -15904,7 +15904,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16" style="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="1" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ration Card, Tier B</t>
+          <t xml:space="preserve">Tier B Rations</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
build(data): Generate World and the content template on main 7819dab
The library lists the house upgrades and effects again and keeps the
radio block over main's portals; a second run changes nothing and
cases.txt is byte-identical. The template carries main's sheets and the
three Home sheets. Every scene rebuilds identically by semantic dump.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -105,6 +105,9 @@
     <sheet name="scriptFonts" sheetId="101" r:id="rId101"/>
     <sheet name="packs" sheetId="102" r:id="rId102"/>
     <sheet name="tongues" sheetId="103" r:id="rId103"/>
+    <sheet name="home" sheetId="104" r:id="rId104"/>
+    <sheet name="homeRadio" sheetId="105" r:id="rId105"/>
+    <sheet name="homeUpgrades" sheetId="106" r:id="rId106"/>
   </sheets>
 </workbook>
 </file>
@@ -15437,6 +15440,509 @@
         </is>
       </c>
     </row>
+    <row r="623">
+      <c r="A623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">home</t>
+        </is>
+      </c>
+      <c r="C623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single</t>
+        </is>
+      </c>
+      <c r="E623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row: the object $.home</t>
+        </is>
+      </c>
+      <c r="F623" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home's house upgrades and the radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">home</t>
+        </is>
+      </c>
+      <c r="B624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">radioUpgrade</t>
+        </is>
+      </c>
+      <c r="C624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F624" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the house upgrade whose ownership plays a radio line on the sleep panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeRadio</t>
+        </is>
+      </c>
+      <c r="C625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.radio, in order</t>
+        </is>
+      </c>
+      <c r="F625" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the radio's lines: one a night, in order by the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeRadio</t>
+        </is>
+      </c>
+      <c r="B626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D626" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="C627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.upgrades, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+      <c r="F627" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the House tree: every effect never takes a knob below 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F628" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the upgrade's id (saved as owned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D629" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">category</t>
+        </is>
+      </c>
+      <c r="C630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: Food, Housing, Security, Health, Comfort</t>
+        </is>
+      </c>
+      <c r="F630" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its column in the House panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B631" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cost</t>
+        </is>
+      </c>
+      <c r="C631" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D631" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F631" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the one-off price in cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B632" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">upkeep</t>
+        </is>
+      </c>
+      <c r="C632" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D632" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F632" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr a night the household pays once it is owned (0: none)</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B633" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requires</t>
+        </is>
+      </c>
+      <c r="C633" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text list</t>
+        </is>
+      </c>
+      <c r="D633" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no items</t>
+        </is>
+      </c>
+      <c r="E633" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">separate items with |</t>
+        </is>
+      </c>
+      <c r="F633" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the house upgrades it needs owned first (ids of this sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B634" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">householdExpense</t>
+        </is>
+      </c>
+      <c r="C634" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D634" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F634" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr a night on rent and utilities (negative saves)</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B635" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sicknessChance</t>
+        </is>
+      </c>
+      <c r="C635" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D635" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F635" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added to each member's nightly chance to worsen (-0.05 = 5 points less)</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B636" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">careCost</t>
+        </is>
+      </c>
+      <c r="C636" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D636" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F636" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr on each treatment (negative cheaper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B637" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medicalDrain</t>
+        </is>
+      </c>
+      <c r="C637" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D637" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F637" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cr on each condition point's nightly drain (negative lowers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B638" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood</t>
+        </is>
+      </c>
+      <c r="C638" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D638" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F638" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the household's mood points (a sick member's nightly recovery chance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B639" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInChance</t>
+        </is>
+      </c>
+      <c r="C639" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D639" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F639" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added to the nightly break-in chance (-0.03 = 3 points less)</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B640" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInShare</t>
+        </is>
+      </c>
+      <c r="C640" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D640" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F640" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added to the share of the wallet a break-in takes</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeUpgrades</t>
+        </is>
+      </c>
+      <c r="B641" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
+      <c r="C641" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D641" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F641" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the House panel's line under its name</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -15714,6 +16220,262 @@
       <c r="E3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">𓄿𓃀𓍿𓂧𓇋𓆑𓎼𓉔𓇌𓆓𓎡𓃭𓅓𓈖𓂝𓊪𓈎𓂋𓋴𓏏𓅱𓎛𓏲𓐍𓏭𓊃</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet104.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">radioUpgrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_radio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet105.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tonight's weather: overcast, with a chance of interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Directorate reminds listeners that sleep is a privilege of the solvent.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet106.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="17" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="8" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">category</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cost</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">upkeep</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requires</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">householdExpense</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sicknessChance</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">careCost</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medicalDrain</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInChance</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">breakInShare</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_rations_b</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tier B Rations</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Food</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>40</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>-0.02</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tier B paste comes in two colours. The kid prefers the green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_veg_box</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vegetable Box</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Food</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>90</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house_rations_b</t>
+        </is>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>-0.04</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Real vegetables, by drone, once a week. The carrots are small, but they are carrots.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
build(endings): generate the world block, rebuild the Title with the world page
- Generate World reads world.factors' answer by name (FactorAnswer; an
  unknown one is an error) in its own partial (WorldContentGenerator.World),
  and writes the world block into ContentLibrary_Main; Strings_en gains
  ending.world.leftBehind; the content spreadsheet template gains the
  worldFactors sheet. Generate World twice: the second run changes nothing.
- Build Title UI adds the world page (heading, the outcomes, the END OF DEMO
  card, New Run with the ending panel's hand-wired face) and the ending
  panel's "The world you leave behind" button; TitleScene rebuilt
  (idempotent by semantic dump). OfficeGameplay is unchanged (its rebuild
  equals the committed scene).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -108,6 +108,7 @@
     <sheet name="home" sheetId="104" r:id="rId104"/>
     <sheet name="homeRadio" sheetId="105" r:id="rId105"/>
     <sheet name="homeUpgrades" sheetId="106" r:id="rId106"/>
+    <sheet name="worldFactors" sheetId="107" r:id="rId107"/>
   </sheets>
 </workbook>
 </file>
@@ -15943,6 +15944,146 @@
         </is>
       </c>
     </row>
+    <row r="642">
+      <c r="A642" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="C642" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E642" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+      <c r="F642" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B643" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C643" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D643" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E643" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F643" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor's id (the endings spec's outcomes name their factor by it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B644" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">question</t>
+        </is>
+      </c>
+      <c r="C644" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D644" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F644" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B645" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">answer</t>
+        </is>
+      </c>
+      <c r="C645" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D645" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E645" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: AsFound, Leader</t>
+        </is>
+      </c>
+      <c r="F645" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads)</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B646" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">foundAs</t>
+        </is>
+      </c>
+      <c r="C646" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D646" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F646" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the answer as the run found 2150</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -16476,6 +16617,86 @@
       <c r="N3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Real vegetables, by drone, once a week. The carrots are small, but they are carrots.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet107.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">question</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">answer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">foundAs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">government</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who runs 2150?</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AsFound</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Directorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What does 2150 run on?</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AsFound</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Credit Age</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(world): rebalance the place leanings and the roles so the demo's world varies (provisional)
The Industrial worksites' leanings spread over several governments and
ways to pay, a few blank cells filled, roles raised (scientist 4, diplomat
and soldier 3, merchant 5). At the shift clock's pace the most frequent
answer now leads 24-34% of careful runs (Monarchy led 54%), every future
and way to pay and every government but Fascism leads in some run, and the
money leaves The Debt in 45-49 of 50 careful runs. Every changed row is in
the endings spec 15.6, provisional for Saleh's review, with the
simulation's before and after.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -18999,7 +18999,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -19014,7 +19014,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -22177,7 +22177,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">monarchy</t>
+          <t xml:space="preserve">theocracy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(paper): the morning paper fits its named headlines; shorter traced lines; the audit asks from the hub and knows a face by its case
The newsletter sheet (briefing and shift report) grows to 860 x 860 and its
body shrinks from 21 to 19 units on a busy day (12.7 px at 720p): the
reference run's day 3 overflowed under Start Shift once its headlines named
the travellers and the desk section told a returning traveller's second
visit. OfficeGameplay rebuilt by Build Office UI (with the wider wheel of
Desk_Default).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -29616,7 +29616,7 @@
     <col min="5" max="5" width="60" style="1" customWidth="1"/>
     <col min="6" max="6" width="60" style="1" customWidth="1"/>
     <col min="7" max="7" width="60" style="1" customWidth="1"/>
-    <col min="8" max="8" width="55" style="1" customWidth="1"/>
+    <col min="8" max="8" width="38" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -29689,17 +29689,17 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">HISTORY: {name}, stamped through Desk 3 on day {day}, brought {value} to {place}.</t>
+          <t xml:space="preserve">HISTORY: {name}, stamped day {day}, brought {value} to {place}.</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PANIC in {place}: {name}, sent through Desk 3 on day {day}, was seen in "{value}" and the street fled.</t>
+          <t xml:space="preserve">PANIC in {place}: {name}, stamped day {day}, wore "{value}". The street fled.</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">It began at Desk 3 with {name}, stamped on day {day}.</t>
+          <t xml:space="preserve">Traced to Desk 3: {name}, day {day}.</t>
         </is>
       </c>
     </row>
@@ -30104,12 +30104,12 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Second time lucky: {name}, turned away at Desk 3 on day {day}, came back on day {back} and was stamped through.</t>
+          <t xml:space="preserve">Second time lucky: {name}, turned away on day {day}, stamped through on day {back}.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">{name} tried Desk 3 again on day {back}, after a refusal on day {day}. Turned away twice.</t>
+          <t xml:space="preserve">{name}, turned away on day {day}, tried again on day {back}. Turned away twice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(history): a front-page story section; 2150 today names its traveller and lists history's changes
StorySection.Front (appended) files a story rule's line on the front page:
it leads the next morning's paper ahead of every other line
(History.FileStory, History.FrontFirst). Chronopedia's present now ends
each "2150 today" answer with the traveller it traces to (Traces.Lines)
and lists history's eight newest changes ("Changed at Desk 3", with the
story rule's name, History.RuleName) before the link to Revisions. The
content sheets accept the new section; the template is rewritten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -14261,12 +14261,12 @@
       </c>
       <c r="E558" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">one of: News, Desk, Return</t>
+          <t xml:space="preserve">one of: News, Desk, Return, Front</t>
         </is>
       </c>
       <c r="F558" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">where the line goes: the paper's news (blank), the paper's desk section, or nowhere until the character returns (its fired flag, trig:history_{id}:fired)</t>
+          <t xml:space="preserve">where the line goes: the paper's news (blank), the paper's desk section, nowhere until the character returns (its fired flag, trig:history_{id}:fired), or the front page, leading the news (a famous traveller's homecoming)</t>
         </is>
       </c>
     </row>
@@ -19261,10 +19261,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="1" customWidth="1"/>
     <col min="6" max="6" width="60" style="1" customWidth="1"/>
   </cols>
@@ -19326,22 +19326,17 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hatshepsut</t>
+          <t xml:space="preserve">senenmut</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hatshepsut</t>
+          <t xml:space="preserve">Senenmut</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">c. 1507 BCE</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1458 BCE</t>
+          <t xml:space="preserve">c. 1505 BCE</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -19351,7 +19346,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pharaoh of Egypt. Senenmut stewarded her household and built her temple.</t>
+          <t xml:space="preserve">Steward of Hatshepsut's household and architect of her temple at Deir el-Bahari.</t>
         </is>
       </c>
     </row>
@@ -30350,16 +30345,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="1" customWidth="1"/>
     <col min="8" max="8" width="60" style="1" customWidth="1"/>
     <col min="9" max="9" width="60" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16" style="1" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="8" style="1" customWidth="1"/>
     <col min="13" max="13" width="8" style="1" customWidth="1"/>
@@ -30453,17 +30448,17 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">senenmut</t>
+          <t xml:space="preserve">hatshepsut</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senenmut</t>
+          <t xml:space="preserve">Hatshepsut</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male</t>
+          <t xml:space="preserve">Female</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -30473,22 +30468,27 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">14 Mar 1505 BCE</t>
+          <t xml:space="preserve">2 Feb 1507 BCE</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">artist</t>
+          <t xml:space="preserve">diplomat</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priority arrival: Hatshepsut, Pharaoh of Egypt. She has brought her own beard.</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steward of the Pharaoh's household and architect of her temple.</t>
+          <t xml:space="preserve">Pharaoh of Upper and Lower Egypt. Wears the royal beard on official business.</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dlg_senenmut</t>
+          <t xml:space="preserve">dlg_hatshepsut</t>
         </is>
       </c>
       <c r="K2" t="b">
@@ -30498,47 +30498,37 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">socrates</t>
+          <t xml:space="preserve">kulthum</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Socrates</t>
+          <t xml:space="preserve">Umm Kulthum</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male</t>
+          <t xml:space="preserve">Female</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">greece_ancient</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">italy_ancient</t>
+          <t xml:space="preserve">egypt_modern</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 Jun 470 BCE</t>
+          <t xml:space="preserve">4 May 1904</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">wanderer</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Priority arrival: Socrates of Athens. He asks more questions than you do.</t>
+          <t xml:space="preserve">artist</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philosopher. Known to question officials at length.</t>
+          <t xml:space="preserve">Singer of Cairo. Her Thursday concerts empty the streets.</t>
         </is>
       </c>
       <c r="K3" t="b">
@@ -30595,9 +30585,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -30626,7 +30616,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">senenmut</t>
+          <t xml:space="preserve">hatshepsut</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -30640,26 +30630,66 @@
         </is>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">socrates</t>
+          <t xml:space="preserve">hatshepsut</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">future</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naturalism</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kulthum</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">money</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commons</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kulthum</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">government</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">democracy</t>
         </is>
       </c>
-      <c r="D3">
+      <c r="D5">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
content: generate the pet's toys (Orders, Toys band), bills and words; the essentials at 28 cr a night after the balance run
Generate World writes the four toys as Orders upgrades with their Mood
effects, the bills and the pet's words into the library's Home content, and
the content template. Food 12, Heating 9, Electricity 7 (the first cut's 24 cr
let 15 of 50 careful climbers reach the top tier at the shift clock's pace;
28 cr brings it back to 1 of 50). The generator's log counts the toys apart.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -123,9 +123,19 @@
     <sheet name="home" sheetId="119" r:id="rId119"/>
     <sheet name="homeRadio" sheetId="120" r:id="rId120"/>
     <sheet name="homeUpgrades" sheetId="121" r:id="rId121"/>
-    <sheet name="worldFactors" sheetId="122" r:id="rId122"/>
-    <sheet name="worldOutcomes" sheetId="123" r:id="rId123"/>
-    <sheet name="worldRoles" sheetId="124" r:id="rId124"/>
+    <sheet name="homeBills" sheetId="122" r:id="rId122"/>
+    <sheet name="homePet" sheetId="123" r:id="rId123"/>
+    <sheet name="homePetKinds" sheetId="124" r:id="rId124"/>
+    <sheet name="homePetReactions" sheetId="125" r:id="rId125"/>
+    <sheet name="homePetToyLines" sheetId="126" r:id="rId126"/>
+    <sheet name="homePetHunger" sheetId="127" r:id="rId127"/>
+    <sheet name="homePetCold" sheetId="128" r:id="rId128"/>
+    <sheet name="homePetBoredom" sheetId="129" r:id="rId129"/>
+    <sheet name="homePetSickness" sheetId="130" r:id="rId130"/>
+    <sheet name="homeToys" sheetId="131" r:id="rId131"/>
+    <sheet name="worldFactors" sheetId="132" r:id="rId132"/>
+    <sheet name="worldOutcomes" sheetId="133" r:id="rId133"/>
+    <sheet name="worldRoles" sheetId="134" r:id="rId134"/>
   </sheets>
 </workbook>
 </file>
@@ -18245,7 +18255,7 @@
       </c>
       <c r="F725" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home's house upgrades and the radio</t>
+          <t xml:space="preserve">Home's house upgrades, the radio, the night's bills, the pet and its toys</t>
         </is>
       </c>
     </row>
@@ -18733,7 +18743,7 @@
     <row r="744">
       <c r="A744" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homeBills</t>
         </is>
       </c>
       <c r="C744" s="1" t="inlineStr">
@@ -18743,24 +18753,24 @@
       </c>
       <c r="E744" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
+          <t xml:space="preserve">one row per item of the list $.home.bills, in order; a row's name is bill, unique</t>
         </is>
       </c>
       <c r="F744" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
+          <t xml:space="preserve">the night's optional bills: the Heating and the TV work only with the Electricity paid</t>
         </is>
       </c>
     </row>
     <row r="745">
       <c r="A745" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homeBills</t>
         </is>
       </c>
       <c r="B745" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">bill</t>
         </is>
       </c>
       <c r="C745" s="1" t="inlineStr">
@@ -18775,24 +18785,24 @@
       </c>
       <c r="E745" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">part of the row's name</t>
+          <t xml:space="preserve">part of the row's name; one of: Food, Heating, Electricity, Tv, Medicine</t>
         </is>
       </c>
       <c r="F745" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor's id (the outcomes, leanings and pulls name their factor by it)</t>
+          <t xml:space="preserve">which of the night's bills (one row each)</t>
         </is>
       </c>
     </row>
     <row r="746">
       <c r="A746" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homeBills</t>
         </is>
       </c>
       <c r="B746" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">question</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="C746" s="1" t="inlineStr">
@@ -18807,51 +18817,46 @@
       </c>
       <c r="F746" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
+          <t xml:space="preserve">its name on the bills panel</t>
         </is>
       </c>
     </row>
     <row r="747">
       <c r="A747" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homeBills</t>
         </is>
       </c>
       <c r="B747" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">answer</t>
+          <t xml:space="preserve">price</t>
         </is>
       </c>
       <c r="C747" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">whole number</t>
         </is>
       </c>
       <c r="D747" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
-        </is>
-      </c>
-      <c r="E747" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one of: AsFound, Leader, Pulls</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="F747" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads); Pulls: the outcome the run's choices pull most (worldOutcomes)</t>
+          <t xml:space="preserve">cr a night (the Medicine's with the house's careCost)</t>
         </is>
       </c>
     </row>
     <row r="748">
       <c r="A748" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homeBills</t>
         </is>
       </c>
       <c r="B748" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">foundAs</t>
+          <t xml:space="preserve">line</t>
         </is>
       </c>
       <c r="C748" s="1" t="inlineStr">
@@ -18861,78 +18866,73 @@
       </c>
       <c r="D748" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F748" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the answer as the run found 2150 (a Pulls factor's is its statusQuo outcome: blank)</t>
+          <t xml:space="preserve">a short line beside it</t>
         </is>
       </c>
     </row>
     <row r="749">
       <c r="A749" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
-        </is>
-      </c>
-      <c r="B749" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">statusQuo</t>
+          <t xml:space="preserve">homePet</t>
         </is>
       </c>
       <c r="C749" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D749" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">Single</t>
+        </is>
+      </c>
+      <c r="E749" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row: the object $.home.pet</t>
         </is>
       </c>
       <c r="F749" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Pulls factor's "as you found it" outcome id: it starts ahead (GameConfigSO worldStatusQuoWeight) and a denial pulls it</t>
+          <t xml:space="preserve">the pet's words: never a number</t>
         </is>
       </c>
     </row>
     <row r="750">
       <c r="A750" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homePet</t>
         </is>
       </c>
       <c r="B750" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">splitLine</t>
+          <t xml:space="preserve">nameMaxLength</t>
         </is>
       </c>
       <c r="C750" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">whole number</t>
         </is>
       </c>
       <c r="D750" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="F750" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Pulls factor's answer when split between two outcomes: {a} and {b} are their names</t>
+          <t xml:space="preserve">the adoption's name limit, in characters</t>
         </is>
       </c>
     </row>
     <row r="751">
       <c r="A751" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">homePet</t>
         </is>
       </c>
       <c r="B751" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">splitHeadline</t>
+          <t xml:space="preserve">worse</t>
         </is>
       </c>
       <c r="C751" s="1" t="inlineStr">
@@ -18942,46 +18942,51 @@
       </c>
       <c r="D751" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F751" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the morning paper's line when the factor splits: {a} and {b}</t>
+          <t xml:space="preserve">Home's line after a night it got sicker</t>
         </is>
       </c>
     </row>
     <row r="752">
       <c r="A752" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">homePet</t>
+        </is>
+      </c>
+      <c r="B752" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">better</t>
         </is>
       </c>
       <c r="C752" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E752" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.outcomes, in order</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D752" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F752" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">every answer of every factor answered by pulls: add rows for more combinations</t>
+          <t xml:space="preserve">Home's line after a night it got better</t>
         </is>
       </c>
     </row>
     <row r="753">
       <c r="A753" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">homePet</t>
         </is>
       </c>
       <c r="B753" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">welfareNotice</t>
         </is>
       </c>
       <c r="C753" s="1" t="inlineStr">
@@ -18991,29 +18996,24 @@
       </c>
       <c r="D753" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
-        </is>
-      </c>
-      <c r="E753" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">names a row of 'worldFactors'</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F753" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor it answers (a Pulls factor)</t>
+          <t xml:space="preserve">Home's warning after a night left at the worst</t>
         </is>
       </c>
     </row>
     <row r="754">
       <c r="A754" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">homePet</t>
         </is>
       </c>
       <c r="B754" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">paperAdopted</t>
         </is>
       </c>
       <c r="C754" s="1" t="inlineStr">
@@ -19023,24 +19023,24 @@
       </c>
       <c r="D754" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F754" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the outcome's id within its factor (leanings and pulls name it)</t>
+          <t xml:space="preserve">the paper the morning after the adoption: {name}, {kind}</t>
         </is>
       </c>
     </row>
     <row r="755">
       <c r="A755" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">homePet</t>
         </is>
       </c>
       <c r="B755" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">paperWelfare</t>
         </is>
       </c>
       <c r="C755" s="1" t="inlineStr">
@@ -19055,46 +19055,36 @@
       </c>
       <c r="F755" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the answer as the player reads it</t>
+          <t xml:space="preserve">the paper after a night left at the worst</t>
         </is>
       </c>
     </row>
     <row r="756">
       <c r="A756" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
-        </is>
-      </c>
-      <c r="B756" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">headline</t>
+          <t xml:space="preserve">homePetKinds</t>
         </is>
       </c>
       <c r="C756" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D756" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">empty text</t>
-        </is>
-      </c>
-      <c r="F756" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the morning paper's line the morning after it takes the lead</t>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E756" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.pet.kinds, in order; a row's name is kind, unique</t>
         </is>
       </c>
     </row>
     <row r="757">
       <c r="A757" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">homePetKinds</t>
         </is>
       </c>
       <c r="B757" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">kind</t>
         </is>
       </c>
       <c r="C757" s="1" t="inlineStr">
@@ -19104,46 +19094,51 @@
       </c>
       <c r="D757" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
-        </is>
-      </c>
-      <c r="F757" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2150 under this answer in a sentence or two, with a joke and an upside, never a verdict</t>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E757" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name; one of: Dog, Cat</t>
         </is>
       </c>
     </row>
     <row r="758">
       <c r="A758" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
+          <t xml:space="preserve">homePetKinds</t>
+        </is>
+      </c>
+      <c r="B758" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">word</t>
         </is>
       </c>
       <c r="C758" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E758" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.roles, in order</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D758" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F758" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">which factor each role pulls; a role not listed pulls nothing</t>
+          <t xml:space="preserve">the kind in a sentence: {kind}</t>
         </is>
       </c>
     </row>
     <row r="759">
       <c r="A759" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
+          <t xml:space="preserve">homePetKinds</t>
         </is>
       </c>
       <c r="B759" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">archetype</t>
+          <t xml:space="preserve">suggestedName</t>
         </is>
       </c>
       <c r="C759" s="1" t="inlineStr">
@@ -19153,69 +19148,971 @@
       </c>
       <c r="D759" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F759" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">an archetype id (content.archetypes)</t>
+          <t xml:space="preserve">the adoption panel's suggestion (a valid name)</t>
         </is>
       </c>
     </row>
     <row r="760">
       <c r="A760" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
-        </is>
-      </c>
-      <c r="B760" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">homePetReactions</t>
         </is>
       </c>
       <c r="C760" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D760" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">Values</t>
         </is>
       </c>
       <c r="E760" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">names a row of 'worldFactors'</t>
+          <t xml:space="preserve">one row per item of the list $.home.pet.kinds[].reactions, in order; the first column names the parent row</t>
         </is>
       </c>
       <c r="F760" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor its accepted travellers pull, toward their destination's leaning</t>
+          <t xml:space="preserve">a pat's lines, in turn: {name}</t>
         </is>
       </c>
     </row>
     <row r="761">
       <c r="A761" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">homePetReactions</t>
+        </is>
+      </c>
+      <c r="B761" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kind</t>
+        </is>
+      </c>
+      <c r="C761" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">row name</t>
+        </is>
+      </c>
+      <c r="D761" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E761" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names the row of 'homePetKinds' this row belongs to</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetReactions</t>
+        </is>
+      </c>
+      <c r="B762" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C762" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D762" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetToyLines</t>
+        </is>
+      </c>
+      <c r="C763" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E763" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.pet.kinds[].toyLines, in order; the first column names the parent row</t>
+        </is>
+      </c>
+      <c r="F763" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a toy's lines, in turn by the day: {name}, {toy}</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetToyLines</t>
+        </is>
+      </c>
+      <c r="B764" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kind</t>
+        </is>
+      </c>
+      <c r="C764" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">row name</t>
+        </is>
+      </c>
+      <c r="D764" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E764" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names the row of 'homePetKinds' this row belongs to</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetToyLines</t>
+        </is>
+      </c>
+      <c r="B765" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C765" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D765" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetHunger</t>
+        </is>
+      </c>
+      <c r="C766" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E766" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.pet.hunger, in order</t>
+        </is>
+      </c>
+      <c r="F766" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hunger in words, best first: {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetHunger</t>
+        </is>
+      </c>
+      <c r="B767" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C767" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D767" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetCold</t>
+        </is>
+      </c>
+      <c r="C768" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E768" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.pet.cold, in order</t>
+        </is>
+      </c>
+      <c r="F768" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cold in words, best first</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetCold</t>
+        </is>
+      </c>
+      <c r="B769" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C769" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D769" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetBoredom</t>
+        </is>
+      </c>
+      <c r="C770" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E770" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.pet.boredom, in order</t>
+        </is>
+      </c>
+      <c r="F770" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">boredom in words, best first</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetBoredom</t>
+        </is>
+      </c>
+      <c r="B771" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C771" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D771" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetSickness</t>
+        </is>
+      </c>
+      <c r="C772" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E772" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.pet.sickness, in order</t>
+        </is>
+      </c>
+      <c r="F772" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sickness in words, best first</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homePetSickness</t>
+        </is>
+      </c>
+      <c r="B773" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C773" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D773" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeToys</t>
+        </is>
+      </c>
+      <c r="C774" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E774" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.home.toys, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeToys</t>
+        </is>
+      </c>
+      <c r="B775" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C775" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D775" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E775" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F775" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the toy's id (an Orders upgrade, saved as owned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeToys</t>
+        </is>
+      </c>
+      <c r="B776" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C776" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D776" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeToys</t>
+        </is>
+      </c>
+      <c r="B777" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cost</t>
+        </is>
+      </c>
+      <c r="C777" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whole number</t>
+        </is>
+      </c>
+      <c r="D777" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F777" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the price in cr at the Orders app</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeToys</t>
+        </is>
+      </c>
+      <c r="B778" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood</t>
+        </is>
+      </c>
+      <c r="C778" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D778" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="F778" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood points while owned (fewer sick nights, quicker recovery)</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">homeToys</t>
+        </is>
+      </c>
+      <c r="B779" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
+      <c r="C779" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D779" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F779" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the Orders app's line</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="C780" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E780" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+      <c r="F780" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B781" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C781" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D781" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E781" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F781" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor's id (the outcomes, leanings and pulls name their factor by it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B782" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">question</t>
+        </is>
+      </c>
+      <c r="C782" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D782" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F782" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B783" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">answer</t>
+        </is>
+      </c>
+      <c r="C783" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D783" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E783" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: AsFound, Leader, Pulls</t>
+        </is>
+      </c>
+      <c r="F783" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads); Pulls: the outcome the run's choices pull most (worldOutcomes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B784" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">foundAs</t>
+        </is>
+      </c>
+      <c r="C784" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D784" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F784" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the answer as the run found 2150 (a Pulls factor's is its statusQuo outcome: blank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B785" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">statusQuo</t>
+        </is>
+      </c>
+      <c r="C785" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D785" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F785" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a Pulls factor's "as you found it" outcome id: it starts ahead (GameConfigSO worldStatusQuoWeight) and a denial pulls it</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B786" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitLine</t>
+        </is>
+      </c>
+      <c r="C786" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D786" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F786" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a Pulls factor's answer when split between two outcomes: {a} and {b} are their names</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B787" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitHeadline</t>
+        </is>
+      </c>
+      <c r="C787" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D787" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F787" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the morning paper's line when the factor splits: {a} and {b}</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="C788" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E788" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.outcomes, in order</t>
+        </is>
+      </c>
+      <c r="F788" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">every answer of every factor answered by pulls: add rows for more combinations</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="C789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'worldFactors'</t>
+        </is>
+      </c>
+      <c r="F789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor it answers (a Pulls factor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B790" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C790" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D790" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="F790" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the outcome's id within its factor (leanings and pulls name it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B791" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C791" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D791" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F791" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the answer as the player reads it</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B792" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">headline</t>
+        </is>
+      </c>
+      <c r="C792" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D792" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F792" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the morning paper's line the morning after it takes the lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
+        </is>
+      </c>
+      <c r="C793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2150 under this answer in a sentence or two, with a joke and an upside, never a verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">worldRoles</t>
         </is>
       </c>
-      <c r="B761" s="1" t="inlineStr">
+      <c r="C794" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E794" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.roles, in order</t>
+        </is>
+      </c>
+      <c r="F794" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">which factor each role pulls; a role not listed pulls nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">archetype</t>
+        </is>
+      </c>
+      <c r="C795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="F795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">an archetype id (content.archetypes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="C796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'worldFactors'</t>
+        </is>
+      </c>
+      <c r="F796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor its accepted travellers pull, toward their destination's leaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B797" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">pull</t>
         </is>
       </c>
-      <c r="C761" s="1" t="inlineStr">
+      <c r="C797" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">number</t>
         </is>
       </c>
-      <c r="D761" s="1" t="inlineStr">
+      <c r="D797" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="F761" s="1" t="inlineStr">
+      <c r="F797" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">one accepted traveller's pull, before the kind's scale (GameConfigSO)</t>
         </is>
@@ -22051,7 +22948,7 @@
       </c>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tier B paste comes in two colours. The kid prefers the green.</t>
+          <t xml:space="preserve">Tier B paste comes in two colours. The pet prefers the green.</t>
         </is>
       </c>
     </row>
@@ -22117,113 +23014,71 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13" style="1" customWidth="1"/>
-    <col min="6" max="6" width="44" style="1" customWidth="1"/>
-    <col min="7" max="7" width="60" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="45" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">bill</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">question</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">answer</t>
+          <t xml:space="preserve">price</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">foundAs</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">statusQuo</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">splitLine</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">splitHeadline</t>
+          <t xml:space="preserve">line</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">government</t>
+          <t xml:space="preserve">Food</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who runs 2150?</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pulls</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">directorate</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{a} and {b}, sharing the building</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TWO GOVERNMENTS: {a} and {b} both claim the Directorate building. Each has opened its own queue.</t>
+          <t xml:space="preserve">Food</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>12</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A night's bowl of Directorate-grade kibble.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">future</t>
+          <t xml:space="preserve">Heating</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">What does 2150 run on?</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pulls</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">credit_age</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{a} and {b}, one on each bank of the river</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2150 IS SPLIT: {a} on one bank of the river, {b} on the other. The bridge is very busy.</t>
+          <t xml:space="preserve">Heating</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The radiator's meter takes credits only.</t>
         </is>
       </c>
     </row>
@@ -22235,91 +23090,73 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="49" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37" style="1" customWidth="1"/>
     <col min="4" max="4" width="60" style="1" customWidth="1"/>
     <col min="5" max="5" width="60" style="1" customWidth="1"/>
+    <col min="6" max="6" width="60" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">nameMaxLength</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">worse</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">better</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">headline</t>
+          <t xml:space="preserve">welfareNotice</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">paperAdopted</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paperWelfare</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">government</t>
-        </is>
+      <c r="A2">
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">directorate</t>
+          <t xml:space="preserve">{name} caught something while you were at work.</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Directorate</t>
+          <t xml:space="preserve">{name} seems brighter this evening.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIRECTORATE: the Customs Directorate carries on running 2150. The queues reopen at nine, as always.</t>
+          <t xml:space="preserve">A notice from the Animal Welfare Office is taped to your door: an inspector will look in on {name} tomorrow night.</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Customs Directorate runs 2150 as it always has: by form, by queue and by stamp. Every citizen knows exactly which counter to stand at.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">government</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">democracy</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Democracy</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2150 VOTES: the Directorate hands the building to an elected assembly. Its first sitting ran eleven hours.</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An elected assembly runs 2150 and votes on everything, including the colour of the ballot papers. Anyone may stand for office, and nearly everyone does.</t>
+          <t xml:space="preserve">SHELTER NEWS: {name} the {kind} has gone home with a clerk of Temporal Customs, Desk 3.</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANIMAL WELFARE: inspectors are asking after a {kind} called {name} in Block C.</t>
         </is>
       </c>
     </row>
@@ -22331,56 +23168,372 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="1" max="1" width="8" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">archetype</t>
+          <t xml:space="preserve">kind</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">word</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">pull</t>
+          <t xml:space="preserve">suggestedName</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">scientist</t>
+          <t xml:space="preserve">Dog</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">future</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>4</v>
+          <t xml:space="preserve">dog</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Biscuit</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">diplomat</t>
+          <t xml:space="preserve">Cat</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">government</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>3</v>
+          <t xml:space="preserve">cat</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Miso</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet125.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8" style="1" customWidth="1"/>
+    <col min="2" max="2" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kind</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} leans into your hand and sighs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name}'s tail thumps the floor twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} rolls over for a belly rub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} licks your wrist, then looks embarrassed about it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} allows it. Briefly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} purrs like a small engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} headbutts your chin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} pretends not to notice, then follows you to the kitchen.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet126.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8" style="1" customWidth="1"/>
+    <col min="2" max="2" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kind</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} carries the {toy} round the flat like a trophy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} drops the {toy} at your feet. Again. And again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dog</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} guards the {toy} from an invisible rival.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} ambushes the {toy} from under the sofa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} bats the {toy} under the radiator and stares at you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cat</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} decides the {toy} is beneath them, then pounces anyway.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet127.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is fed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is hungry.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet128.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is warm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is chilly.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet129.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is playful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is restless.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -22460,6 +23613,400 @@
         <v>0</v>
       </c>
       <c r="E3">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet130.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is healthy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name} is a little unwell.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet131.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cost</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mood</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blurb</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">toy_ball</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pre-owned Tennis Ball</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Slightly bald. It bounces in 2150 the way it bounced in 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">toy_rope</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rope of Regulation Length</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Certified tug-worthy by the Bureau of Standards. Chewing voids the warranty.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet132.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13" style="1" customWidth="1"/>
+    <col min="6" max="6" width="44" style="1" customWidth="1"/>
+    <col min="7" max="7" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">question</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">answer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">foundAs</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">statusQuo</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitLine</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitHeadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">government</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who runs 2150?</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulls</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">directorate</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{a} and {b}, sharing the building</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TWO GOVERNMENTS: {a} and {b} both claim the Directorate building. Each has opened its own queue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What does 2150 run on?</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulls</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">credit_age</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{a} and {b}, one on each bank of the river</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2150 IS SPLIT: {a} on one bank of the river, {b} on the other. The bridge is very busy.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17" style="1" customWidth="1"/>
+    <col min="4" max="4" width="60" style="1" customWidth="1"/>
+    <col min="5" max="5" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">headline</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">government</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">directorate</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Directorate</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIRECTORATE: the Customs Directorate carries on running 2150. The queues reopen at nine, as always.</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Customs Directorate runs 2150 as it always has: by form, by queue and by stamp. Every citizen knows exactly which counter to stand at.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">government</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">democracy</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Democracy</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2150 VOTES: the Directorate hands the building to an elected assembly. Its first sitting ran eleven hours.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An elected assembly runs 2150 and votes on everything, including the colour of the ballot papers. Anyone may stand for office, and nearly everyone does.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet134.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">archetype</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pull</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scientist</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">future</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">diplomat</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">government</t>
+        </is>
+      </c>
+      <c r="C3">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
content: the content template rewritten after the merge (the pet's sheets with main's)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -14271,12 +14271,12 @@
       </c>
       <c r="E558" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">one of: News, Desk, Return</t>
+          <t xml:space="preserve">one of: News, Desk, Return, Front</t>
         </is>
       </c>
       <c r="F558" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">where the line goes: the paper's news (blank), the paper's desk section, or nowhere until the character returns (its fired flag, trig:history_{id}:fired)</t>
+          <t xml:space="preserve">where the line goes: the paper's news (blank), the paper's desk section, nowhere until the character returns (its fired flag, trig:history_{id}:fired), or the front page, leading the news (a famous traveller's homecoming)</t>
         </is>
       </c>
     </row>
@@ -20158,10 +20158,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="1" customWidth="1"/>
     <col min="6" max="6" width="60" style="1" customWidth="1"/>
   </cols>
@@ -20223,22 +20223,17 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hatshepsut</t>
+          <t xml:space="preserve">senenmut</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hatshepsut</t>
+          <t xml:space="preserve">Senenmut</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">c. 1507 BCE</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1458 BCE</t>
+          <t xml:space="preserve">c. 1505 BCE</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -20248,7 +20243,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pharaoh of Egypt. Senenmut stewarded her household and built her temple.</t>
+          <t xml:space="preserve">Steward of Hatshepsut's household and architect of her temple at Deir el-Bahari.</t>
         </is>
       </c>
     </row>
@@ -31897,16 +31892,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="1" customWidth="1"/>
     <col min="8" max="8" width="60" style="1" customWidth="1"/>
     <col min="9" max="9" width="60" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16" style="1" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="8" style="1" customWidth="1"/>
     <col min="13" max="13" width="8" style="1" customWidth="1"/>
@@ -32000,17 +31995,17 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">senenmut</t>
+          <t xml:space="preserve">hatshepsut</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senenmut</t>
+          <t xml:space="preserve">Hatshepsut</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male</t>
+          <t xml:space="preserve">Female</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -32020,22 +32015,27 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">14 Mar 1505 BCE</t>
+          <t xml:space="preserve">2 Feb 1507 BCE</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">artist</t>
+          <t xml:space="preserve">diplomat</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priority arrival: Hatshepsut, Pharaoh of Egypt. She has brought her own beard.</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steward of the Pharaoh's household and architect of her temple.</t>
+          <t xml:space="preserve">Pharaoh of Upper and Lower Egypt. Wears the royal beard on official business.</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dlg_senenmut</t>
+          <t xml:space="preserve">dlg_hatshepsut</t>
         </is>
       </c>
       <c r="K2" t="b">
@@ -32045,47 +32045,37 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">socrates</t>
+          <t xml:space="preserve">kulthum</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Socrates</t>
+          <t xml:space="preserve">Umm Kulthum</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male</t>
+          <t xml:space="preserve">Female</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">greece_ancient</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">italy_ancient</t>
+          <t xml:space="preserve">egypt_modern</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 Jun 470 BCE</t>
+          <t xml:space="preserve">4 May 1904</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">wanderer</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Priority arrival: Socrates of Athens. He asks more questions than you do.</t>
+          <t xml:space="preserve">artist</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philosopher. Known to question officials at length.</t>
+          <t xml:space="preserve">Singer of Cairo. Her Thursday concerts empty the streets.</t>
         </is>
       </c>
       <c r="K3" t="b">
@@ -32142,7 +32132,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="1" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
@@ -32173,7 +32163,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">senenmut</t>
+          <t xml:space="preserve">hatshepsut</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -32187,26 +32177,66 @@
         </is>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">socrates</t>
+          <t xml:space="preserve">hatshepsut</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">money</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jubilee</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kulthum</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">money</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commons</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kulthum</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">government</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">democracy</t>
         </is>
       </c>
-      <c r="D3">
+      <c r="D5">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(documents): a plain passport and short agency numbers
Saleh 2026-10-06: "there is a long number on the passport and many <<<<.
I know this is how it looks in real life but it is confusing to the
player; let's simplify, look at the fields in Papers, Please."
- The passport's machine-readable zone is gone (MachineZone, its tests,
  the Mrz block kind 18, its metrics and text role; 18 is never reused);
  the nation's three-letter code prints under the emblem instead.
- Every compared agency number is short: a Citizen ID "KTR-418" (three
  capitals without I and O, three digits; three draws as before), a
  Displacement No. "DP-4471", a waiver or policy number "SW-2048" /
  "TI-5519". The authored IDs in world_source.json are rewritten; Generate
  World, the validator and the content sheet notes take the new format.
- FEATURES: Papers, Travel documents and the examples' numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -3765,7 +3765,7 @@
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three-letter code the passport's machine-readable zone prints (EGY)</t>
+          <t xml:space="preserve">the three-letter code the passport prints under its emblem (EGY)</t>
         </is>
       </c>
     </row>
@@ -13730,7 +13730,7 @@
       </c>
       <c r="F535" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">a story character's Citizen ID (000-0000-00), the same at every appearance</t>
+          <t xml:space="preserve">a story character's Citizen ID (AAA-000: three capitals but I and O, three digits), the same at every appearance</t>
         </is>
       </c>
     </row>
@@ -21170,7 +21170,7 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">773-2840-19</t>
+          <t xml:space="preserve">TMW-773</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
content: the guide's words: BASICS, a page per introduced feature, day 1's steps
world_source.json "guide" (the BASICS lines, 18 pages keyed by their
Introductions feature with where the moment points and the guided days'
practices, the eight FTUE steps, the closing line, guidedThroughDay 7)
and the guide's ui strings; Generate World checks it against the ramp
(GuideContent.Problems) and writes ContentLibrarySO.Guide; the validator
checks the same; content sheets guide, guideBasics, guidePages,
guideFtue; the narrative workbook's "The desk's guide" block.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -133,9 +133,13 @@
     <sheet name="homePetBoredom" sheetId="129" r:id="rId129"/>
     <sheet name="homePetSickness" sheetId="130" r:id="rId130"/>
     <sheet name="homeToys" sheetId="131" r:id="rId131"/>
-    <sheet name="worldFactors" sheetId="132" r:id="rId132"/>
-    <sheet name="worldOutcomes" sheetId="133" r:id="rId133"/>
-    <sheet name="worldRoles" sheetId="134" r:id="rId134"/>
+    <sheet name="guide" sheetId="132" r:id="rId132"/>
+    <sheet name="guideBasics" sheetId="133" r:id="rId133"/>
+    <sheet name="guidePages" sheetId="134" r:id="rId134"/>
+    <sheet name="guideFtue" sheetId="135" r:id="rId135"/>
+    <sheet name="worldFactors" sheetId="136" r:id="rId136"/>
+    <sheet name="worldOutcomes" sheetId="137" r:id="rId137"/>
+    <sheet name="worldRoles" sheetId="138" r:id="rId138"/>
   </sheets>
 </workbook>
 </file>
@@ -19780,66 +19784,61 @@
     <row r="785">
       <c r="A785" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guide</t>
         </is>
       </c>
       <c r="C785" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
+          <t xml:space="preserve">Single</t>
         </is>
       </c>
       <c r="E785" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
+          <t xml:space="preserve">one row: the object $.guide</t>
         </is>
       </c>
       <c r="F785" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
+          <t xml:space="preserve">the FTUE and the rulebook's GUIDE pages</t>
         </is>
       </c>
     </row>
     <row r="786">
       <c r="A786" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guide</t>
         </is>
       </c>
       <c r="B786" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">guidedThroughDay</t>
         </is>
       </c>
       <c r="C786" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">whole number</t>
         </is>
       </c>
       <c r="D786" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
-        </is>
-      </c>
-      <c r="E786" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">part of the row's name</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="F786" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor's id (the outcomes, leanings and pulls name their factor by it)</t>
+          <t xml:space="preserve">the last day the rulebook opens itself on the day's new page with a practice prompt; later days only badge the GUIDE tab</t>
         </is>
       </c>
     </row>
     <row r="787">
       <c r="A787" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guide</t>
         </is>
       </c>
       <c r="B787" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">question</t>
+          <t xml:space="preserve">basicsTitle</t>
         </is>
       </c>
       <c r="C787" s="1" t="inlineStr">
@@ -19854,19 +19853,19 @@
       </c>
       <c r="F787" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
+          <t xml:space="preserve">the BASICS page's heading</t>
         </is>
       </c>
     </row>
     <row r="788">
       <c r="A788" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guide</t>
         </is>
       </c>
       <c r="B788" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">answer</t>
+          <t xml:space="preserve">ftueDone</t>
         </is>
       </c>
       <c r="C788" s="1" t="inlineStr">
@@ -19879,53 +19878,43 @@
           <t xml:space="preserve">empty text</t>
         </is>
       </c>
-      <c r="E788" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one of: AsFound, Leader, Pulls</t>
-        </is>
-      </c>
       <c r="F788" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads); Pulls: the outcome the run's choices pull most (worldOutcomes)</t>
+          <t xml:space="preserve">the line once the last step is done</t>
         </is>
       </c>
     </row>
     <row r="789">
       <c r="A789" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
-        </is>
-      </c>
-      <c r="B789" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">foundAs</t>
+          <t xml:space="preserve">guideBasics</t>
         </is>
       </c>
       <c r="C789" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D789" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">Values</t>
+        </is>
+      </c>
+      <c r="E789" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.guide.basics, in order</t>
         </is>
       </c>
       <c r="F789" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the answer as the run found 2150 (a Pulls factor's is its statusQuo outcome: blank)</t>
+          <t xml:space="preserve">the BASICS page's lines, in order: {inspect}, {stamps}, {pc}, {back} print the keys</t>
         </is>
       </c>
     </row>
     <row r="790">
       <c r="A790" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guideBasics</t>
         </is>
       </c>
       <c r="B790" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">statusQuo</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="C790" s="1" t="inlineStr">
@@ -19935,51 +19924,41 @@
       </c>
       <c r="D790" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
-        </is>
-      </c>
-      <c r="F790" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a Pulls factor's "as you found it" outcome id: it starts ahead (GameConfigSO worldStatusQuoWeight) and a denial pulls it</t>
+          <t xml:space="preserve">(required)</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
-        </is>
-      </c>
-      <c r="B791" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">splitLine</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="C791" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D791" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E791" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.guide.pages, in order; a row's name is id, unique</t>
         </is>
       </c>
       <c r="F791" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Pulls factor's answer when split between two outcomes: {a} and {b} are their names</t>
+          <t xml:space="preserve">one page per introduced paper, rule or tool, added the day its feature is introduced (Introductions)</t>
         </is>
       </c>
     </row>
     <row r="792">
       <c r="A792" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B792" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">splitHeadline</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="C792" s="1" t="inlineStr">
@@ -19989,46 +19968,56 @@
       </c>
       <c r="D792" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E792" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
         </is>
       </c>
       <c r="F792" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the morning paper's line when the factor splits: {a} and {b}</t>
+          <t xml:space="preserve">the page's id (saved as read and practised)</t>
         </is>
       </c>
     </row>
     <row r="793">
       <c r="A793" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">guidePages</t>
+        </is>
+      </c>
+      <c r="B793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature</t>
         </is>
       </c>
       <c r="C793" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E793" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.outcomes, in order</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D793" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
         </is>
       </c>
       <c r="F793" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">every answer of every factor answered by pulls: add rows for more combinations</t>
+          <t xml:space="preserve">the introduction key that adds the page on its first day: paper:TC-230, tool:board, book:Seal, rule:Rule_DebtStanding</t>
         </is>
       </c>
     </row>
     <row r="794">
       <c r="A794" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B794" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">title</t>
         </is>
       </c>
       <c r="C794" s="1" t="inlineStr">
@@ -20038,29 +20027,24 @@
       </c>
       <c r="D794" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
-        </is>
-      </c>
-      <c r="E794" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">names a row of 'worldFactors'</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F794" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor it answers (a Pulls factor)</t>
+          <t xml:space="preserve">the page's heading</t>
         </is>
       </c>
     </row>
     <row r="795">
       <c r="A795" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B795" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">check</t>
         </is>
       </c>
       <c r="C795" s="1" t="inlineStr">
@@ -20070,24 +20054,24 @@
       </c>
       <c r="D795" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F795" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the outcome's id within its factor (leanings and pulls name it)</t>
+          <t xml:space="preserve">what to check</t>
         </is>
       </c>
     </row>
     <row r="796">
       <c r="A796" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B796" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">against</t>
         </is>
       </c>
       <c r="C796" s="1" t="inlineStr">
@@ -20102,19 +20086,19 @@
       </c>
       <c r="F796" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the answer as the player reads it</t>
+          <t xml:space="preserve">what to check it against</t>
         </is>
       </c>
     </row>
     <row r="797">
       <c r="A797" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B797" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">headline</t>
+          <t xml:space="preserve">fault</t>
         </is>
       </c>
       <c r="C797" s="1" t="inlineStr">
@@ -20129,19 +20113,19 @@
       </c>
       <c r="F797" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the morning paper's line the morning after it takes the lead</t>
+          <t xml:space="preserve">an example of a fault</t>
         </is>
       </c>
     </row>
     <row r="798">
       <c r="A798" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B798" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">point</t>
         </is>
       </c>
       <c r="C798" s="1" t="inlineStr">
@@ -20156,41 +20140,46 @@
       </c>
       <c r="F798" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2150 under this answer in a sentence or two, with a joke and an upside, never a verdict</t>
+          <t xml:space="preserve">where the new rule's moment points: sign, inspect, stamps, pc, rulebook, calendar, board, scanner, counter, traveller, paper:&lt;form&gt;, field:&lt;form&gt;/&lt;detail&gt;</t>
         </is>
       </c>
     </row>
     <row r="799">
       <c r="A799" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
+          <t xml:space="preserve">guidePages</t>
+        </is>
+      </c>
+      <c r="B799" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.id</t>
         </is>
       </c>
       <c r="C799" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E799" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.roles, in order</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D799" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F799" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">which factor each role pulls; a role not listed pulls nothing</t>
+          <t xml:space="preserve">the practice's id (blank: no practice)</t>
         </is>
       </c>
     </row>
     <row r="800">
       <c r="A800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">archetype</t>
+          <t xml:space="preserve">practice.action</t>
         </is>
       </c>
       <c r="C800" s="1" t="inlineStr">
@@ -20200,69 +20189,818 @@
       </c>
       <c r="D800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E800" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: , Call, OnDesk, Inspect, Compare, StampsOut, Stamp, HandBack, Scan</t>
         </is>
       </c>
       <c r="F800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">an archetype id (content.archetypes)</t>
+          <t xml:space="preserve">what completes the practice on the first traveller who carries the page's feature (blank: no practice)</t>
         </is>
       </c>
     </row>
     <row r="801">
       <c r="A801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
+          <t xml:space="preserve">guidePages</t>
         </is>
       </c>
       <c r="B801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">practice.categories</t>
         </is>
       </c>
       <c r="C801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">text list</t>
         </is>
       </c>
       <c r="D801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">no items</t>
         </is>
       </c>
       <c r="E801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">names a row of 'worldFactors'</t>
+          <t xml:space="preserve">separate items with |</t>
         </is>
       </c>
       <c r="F801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor its accepted travellers pull, toward their destination's leaning</t>
+          <t xml:space="preserve">for Compare: the details the comparison must be about, any of them (blank: any)</t>
         </is>
       </c>
     </row>
     <row r="802">
       <c r="A802" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">guidePages</t>
+        </is>
+      </c>
+      <c r="B802" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.form</t>
+        </is>
+      </c>
+      <c r="C802" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D802" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F802" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">for OnDesk: the paper's form (blank: any)</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guidePages</t>
+        </is>
+      </c>
+      <c r="B803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.target</t>
+        </is>
+      </c>
+      <c r="C803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">where the practice's arrow points (as point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guidePages</t>
+        </is>
+      </c>
+      <c r="B804" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.text</t>
+        </is>
+      </c>
+      <c r="C804" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D804" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F804" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the practice prompt's line: {inspect}, {stamps}, {pc}, {back} print the keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="C805" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E805" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.guide.ftue, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+      <c r="F805" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">day 1's steps, in order: each completes when the player does its action</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the step's id (saved as done)</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">action</t>
+        </is>
+      </c>
+      <c r="C807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: Call, OnDesk, Inspect, Compare, StampsOut, Stamp, HandBack, Scan</t>
+        </is>
+      </c>
+      <c r="F807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">what the player does to complete it</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B808" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">categories</t>
+        </is>
+      </c>
+      <c r="C808" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text list</t>
+        </is>
+      </c>
+      <c r="D808" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no items</t>
+        </is>
+      </c>
+      <c r="E808" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">separate items with |</t>
+        </is>
+      </c>
+      <c r="F808" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">for Compare: the details the comparison must be about, any of them (blank: any)</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">form</t>
+        </is>
+      </c>
+      <c r="C809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">for OnDesk: the paper's form (blank: any)</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B810" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target</t>
+        </is>
+      </c>
+      <c r="C810" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D810" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F810" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">where the arrow points (as guidePages.point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B811" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="C811" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D811" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F811" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the prompt's one line: {inspect}, {stamps}, {pc}, {back} print the keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="C812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
+        </is>
+      </c>
+      <c r="F812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B813" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C813" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D813" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E813" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
+        </is>
+      </c>
+      <c r="F813" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor's id (the outcomes, leanings and pulls name their factor by it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">question</t>
+        </is>
+      </c>
+      <c r="C814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B815" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">answer</t>
+        </is>
+      </c>
+      <c r="C815" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D815" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E815" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: AsFound, Leader, Pulls</t>
+        </is>
+      </c>
+      <c r="F815" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads); Pulls: the outcome the run's choices pull most (worldOutcomes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B816" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">foundAs</t>
+        </is>
+      </c>
+      <c r="C816" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D816" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F816" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the answer as the run found 2150 (a Pulls factor's is its statusQuo outcome: blank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B817" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">statusQuo</t>
+        </is>
+      </c>
+      <c r="C817" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D817" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F817" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a Pulls factor's "as you found it" outcome id: it starts ahead (GameConfigSO worldStatusQuoWeight) and a denial pulls it</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B818" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitLine</t>
+        </is>
+      </c>
+      <c r="C818" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D818" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F818" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a Pulls factor's answer when split between two outcomes: {a} and {b} are their names</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B819" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitHeadline</t>
+        </is>
+      </c>
+      <c r="C819" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D819" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
+        </is>
+      </c>
+      <c r="F819" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the morning paper's line when the factor splits: {a} and {b}</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="C820" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E820" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.outcomes, in order</t>
+        </is>
+      </c>
+      <c r="F820" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">every answer of every factor answered by pulls: add rows for more combinations</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B821" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="C821" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D821" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E821" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'worldFactors'</t>
+        </is>
+      </c>
+      <c r="F821" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor it answers (a Pulls factor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B822" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="C822" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D822" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="F822" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the outcome's id within its factor (leanings and pulls name it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B823" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C823" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D823" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F823" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the answer as the player reads it</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B824" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">headline</t>
+        </is>
+      </c>
+      <c r="C824" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D824" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F824" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the morning paper's line the morning after it takes the lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B825" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
+        </is>
+      </c>
+      <c r="C825" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D825" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="F825" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2150 under this answer in a sentence or two, with a joke and an upside, never a verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">worldRoles</t>
         </is>
       </c>
-      <c r="B802" s="1" t="inlineStr">
+      <c r="C826" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E826" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.roles, in order</t>
+        </is>
+      </c>
+      <c r="F826" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">which factor each role pulls; a role not listed pulls nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B827" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">archetype</t>
+        </is>
+      </c>
+      <c r="C827" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D827" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="F827" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">an archetype id (content.archetypes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B828" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="C828" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D828" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E828" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'worldFactors'</t>
+        </is>
+      </c>
+      <c r="F828" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor its accepted travellers pull, toward their destination's leaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B829" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">pull</t>
         </is>
       </c>
-      <c r="C802" s="1" t="inlineStr">
+      <c r="C829" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">number</t>
         </is>
       </c>
-      <c r="D802" s="1" t="inlineStr">
+      <c r="D829" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="F802" s="1" t="inlineStr">
+      <c r="F829" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">one accepted traveller's pull, before the kind's scale (GameConfigSO)</t>
         </is>
@@ -23894,6 +24632,339 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="13" style="1" customWidth="1"/>
+    <col min="3" max="3" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guidedThroughDay</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">basicsTitle</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ftueDone</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BASICS</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">That is the job. The rulebook's GUIDE tab explains every rule, and new rules add new pages. F1 lists the keys.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Left-drag moves a paper: small on the counter, full size on the desk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{inspect} or the red magnifier: inspect. Click one value, then another, to compare them.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet134.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29" style="1" customWidth="1"/>
+    <col min="5" max="5" width="60" style="1" customWidth="1"/>
+    <col min="6" max="6" width="57" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15" style="1" customWidth="1"/>
+    <col min="12" max="12" width="17" style="1" customWidth="1"/>
+    <col min="13" max="13" width="15" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feature</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">title</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">check</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">against</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fault</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">point</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.id</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.action</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.categories</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.form</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.target</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">passport</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paper:TC-101</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THE PASSPORT</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Its photo and its name.</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The traveller at the desk: is it their face?</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Someone else's photo: deny.</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paper:TC-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">destination</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tool:rulebook</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TODAY'S DESTINATION</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Passport's Destination.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Today's rule on the RULES tab (from day 3 the Departure Board shows it too).</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Republican Rome on a day only Periclean Athens is open.</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rulebook</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet135.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="1" customWidth="1"/>
+    <col min="6" max="6" width="60" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">action</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">categories</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">form</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">call</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Call</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sign</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Click the AVAILABLE sign to call the first traveller.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">desk</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OnDesk</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paper:TC-101</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drag the Passport from the counter onto the desk to read it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet136.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
     <col min="2" max="2" width="24" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" customWidth="1"/>
@@ -24008,7 +25079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet137.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -24104,7 +25175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet134.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet138.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
feat(desk): the Seal Register at the desk, and the tutorial's prompt at the top left
The rulebook's fourth tab, SEALS (from day 4, Feature.Book(Seal)): a row
per issuing office with its seal and name, comparable in inspect mode
through the PC register's compare (EvidencePicks.ForSeal), so day 4's
seals are checked at the desk and its page has its practice; the PC's
register stays. The guide's prompt moves to the top left, clear of the
papers and the rulebook in the reading view. OfficeGameplay rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -20044,7 +20044,7 @@
       </c>
       <c r="B795" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">check</t>
+          <t xml:space="preserve">named</t>
         </is>
       </c>
       <c r="C795" s="1" t="inlineStr">
@@ -20059,7 +20059,7 @@
       </c>
       <c r="F795" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">what to check</t>
+          <t xml:space="preserve">the words the bulletin of the page's day names it by (any case; Generate World refuses a bulletin without them)</t>
         </is>
       </c>
     </row>
@@ -20071,7 +20071,7 @@
       </c>
       <c r="B796" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">against</t>
+          <t xml:space="preserve">check</t>
         </is>
       </c>
       <c r="C796" s="1" t="inlineStr">
@@ -20086,7 +20086,7 @@
       </c>
       <c r="F796" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">what to check it against</t>
+          <t xml:space="preserve">what to check</t>
         </is>
       </c>
     </row>
@@ -20098,7 +20098,7 @@
       </c>
       <c r="B797" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">fault</t>
+          <t xml:space="preserve">against</t>
         </is>
       </c>
       <c r="C797" s="1" t="inlineStr">
@@ -20113,7 +20113,7 @@
       </c>
       <c r="F797" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">an example of a fault</t>
+          <t xml:space="preserve">what to check it against</t>
         </is>
       </c>
     </row>
@@ -20125,7 +20125,7 @@
       </c>
       <c r="B798" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">point</t>
+          <t xml:space="preserve">fault</t>
         </is>
       </c>
       <c r="C798" s="1" t="inlineStr">
@@ -20140,7 +20140,7 @@
       </c>
       <c r="F798" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">where the new rule's moment points: sign, inspect, stamps, pc, rulebook, calendar, board, scanner, counter, traveller, paper:&lt;form&gt;, field:&lt;form&gt;/&lt;detail&gt;</t>
+          <t xml:space="preserve">an example of a fault</t>
         </is>
       </c>
     </row>
@@ -20152,7 +20152,7 @@
       </c>
       <c r="B799" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">practice.id</t>
+          <t xml:space="preserve">point</t>
         </is>
       </c>
       <c r="C799" s="1" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="F799" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the practice's id (blank: no practice)</t>
+          <t xml:space="preserve">where the new rule's moment points: sign, inspect, stamps, pc, rulebook, calendar, board, scanner, counter, traveller, paper:&lt;form&gt;, field:&lt;form&gt;/&lt;detail&gt;</t>
         </is>
       </c>
     </row>
@@ -20179,7 +20179,7 @@
       </c>
       <c r="B800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">practice.action</t>
+          <t xml:space="preserve">practice.id</t>
         </is>
       </c>
       <c r="C800" s="1" t="inlineStr">
@@ -20192,14 +20192,9 @@
           <t xml:space="preserve">empty text</t>
         </is>
       </c>
-      <c r="E800" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one of: , Call, OnDesk, Inspect, Compare, StampsOut, Stamp, HandBack, Scan</t>
-        </is>
-      </c>
       <c r="F800" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">what completes the practice on the first traveller who carries the page's feature (blank: no practice)</t>
+          <t xml:space="preserve">the practice's id (blank: no practice)</t>
         </is>
       </c>
     </row>
@@ -20211,27 +20206,27 @@
       </c>
       <c r="B801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">practice.categories</t>
+          <t xml:space="preserve">practice.action</t>
         </is>
       </c>
       <c r="C801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text list</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">no items</t>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="E801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">separate items with |</t>
+          <t xml:space="preserve">one of: , Call, OnDesk, Inspect, Compare, StampsOut, Stamp, HandBack, Scan</t>
         </is>
       </c>
       <c r="F801" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">for Compare: the details the comparison must be about, any of them (blank: any)</t>
+          <t xml:space="preserve">what completes the practice on the first traveller who carries the page's feature (blank: no practice)</t>
         </is>
       </c>
     </row>
@@ -20243,22 +20238,27 @@
       </c>
       <c r="B802" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">practice.form</t>
+          <t xml:space="preserve">practice.categories</t>
         </is>
       </c>
       <c r="C802" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">text list</t>
         </is>
       </c>
       <c r="D802" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">no items</t>
+        </is>
+      </c>
+      <c r="E802" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">separate items with |</t>
         </is>
       </c>
       <c r="F802" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">for OnDesk: the paper's form (blank: any)</t>
+          <t xml:space="preserve">for Compare: the details the comparison must be about, any of them (blank: any)</t>
         </is>
       </c>
     </row>
@@ -20270,7 +20270,7 @@
       </c>
       <c r="B803" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">practice.target</t>
+          <t xml:space="preserve">practice.form</t>
         </is>
       </c>
       <c r="C803" s="1" t="inlineStr">
@@ -20285,7 +20285,7 @@
       </c>
       <c r="F803" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">where the practice's arrow points (as point)</t>
+          <t xml:space="preserve">for OnDesk: the paper's form (blank: any)</t>
         </is>
       </c>
     </row>
@@ -20297,7 +20297,7 @@
       </c>
       <c r="B804" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">practice.text</t>
+          <t xml:space="preserve">practice.target</t>
         </is>
       </c>
       <c r="C804" s="1" t="inlineStr">
@@ -20312,29 +20312,34 @@
       </c>
       <c r="F804" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the practice prompt's line: {inspect}, {stamps}, {pc}, {back} print the keys</t>
+          <t xml:space="preserve">where the practice's arrow points (as point)</t>
         </is>
       </c>
     </row>
     <row r="805">
       <c r="A805" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">guideFtue</t>
+          <t xml:space="preserve">guidePages</t>
+        </is>
+      </c>
+      <c r="B805" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">practice.text</t>
         </is>
       </c>
       <c r="C805" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E805" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.guide.ftue, in order; a row's name is id, unique</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D805" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F805" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">day 1's steps, in order: each completes when the player does its action</t>
+          <t xml:space="preserve">the practice prompt's line: {inspect}, {stamps}, {pc}, {back} print the keys</t>
         </is>
       </c>
     </row>
@@ -20344,29 +20349,19 @@
           <t xml:space="preserve">guideFtue</t>
         </is>
       </c>
-      <c r="B806" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
       <c r="C806" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D806" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">Rows</t>
         </is>
       </c>
       <c r="E806" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">part of the row's name</t>
+          <t xml:space="preserve">one row per item of the list $.guide.ftue, in order; a row's name is id, unique</t>
         </is>
       </c>
       <c r="F806" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the step's id (saved as done)</t>
+          <t xml:space="preserve">day 1's steps, in order: each completes when the player does its action</t>
         </is>
       </c>
     </row>
@@ -20378,7 +20373,7 @@
       </c>
       <c r="B807" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">action</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="C807" s="1" t="inlineStr">
@@ -20393,12 +20388,12 @@
       </c>
       <c r="E807" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">one of: Call, OnDesk, Inspect, Compare, StampsOut, Stamp, HandBack, Scan</t>
+          <t xml:space="preserve">part of the row's name</t>
         </is>
       </c>
       <c r="F807" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the player does to complete it</t>
+          <t xml:space="preserve">the step's id (saved as done)</t>
         </is>
       </c>
     </row>
@@ -20410,27 +20405,27 @@
       </c>
       <c r="B808" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">categories</t>
+          <t xml:space="preserve">action</t>
         </is>
       </c>
       <c r="C808" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text list</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D808" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">no items</t>
+          <t xml:space="preserve">(required)</t>
         </is>
       </c>
       <c r="E808" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">separate items with |</t>
+          <t xml:space="preserve">one of: Call, OnDesk, Inspect, Compare, StampsOut, Stamp, HandBack, Scan</t>
         </is>
       </c>
       <c r="F808" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">for Compare: the details the comparison must be about, any of them (blank: any)</t>
+          <t xml:space="preserve">what the player does to complete it</t>
         </is>
       </c>
     </row>
@@ -20442,22 +20437,27 @@
       </c>
       <c r="B809" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">form</t>
+          <t xml:space="preserve">categories</t>
         </is>
       </c>
       <c r="C809" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">text list</t>
         </is>
       </c>
       <c r="D809" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">no items</t>
+        </is>
+      </c>
+      <c r="E809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">separate items with |</t>
         </is>
       </c>
       <c r="F809" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">for OnDesk: the paper's form (blank: any)</t>
+          <t xml:space="preserve">for Compare: the details the comparison must be about, any of them (blank: any)</t>
         </is>
       </c>
     </row>
@@ -20469,7 +20469,7 @@
       </c>
       <c r="B810" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">target</t>
+          <t xml:space="preserve">form</t>
         </is>
       </c>
       <c r="C810" s="1" t="inlineStr">
@@ -20484,7 +20484,7 @@
       </c>
       <c r="F810" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">where the arrow points (as guidePages.point)</t>
+          <t xml:space="preserve">for OnDesk: the paper's form (blank: any)</t>
         </is>
       </c>
     </row>
@@ -20496,7 +20496,7 @@
       </c>
       <c r="B811" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">target</t>
         </is>
       </c>
       <c r="C811" s="1" t="inlineStr">
@@ -20511,29 +20511,34 @@
       </c>
       <c r="F811" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the prompt's one line: {inspect}, {stamps}, {pc}, {back} print the keys</t>
+          <t xml:space="preserve">where the arrow points (as guidePages.point)</t>
         </is>
       </c>
     </row>
     <row r="812">
       <c r="A812" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldFactors</t>
+          <t xml:space="preserve">guideFtue</t>
+        </is>
+      </c>
+      <c r="B812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="C812" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E812" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F812" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
+          <t xml:space="preserve">the prompt's one line: {inspect}, {stamps}, {pc}, {back} print the keys</t>
         </is>
       </c>
     </row>
@@ -20543,29 +20548,19 @@
           <t xml:space="preserve">worldFactors</t>
         </is>
       </c>
-      <c r="B813" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
       <c r="C813" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D813" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">Rows</t>
         </is>
       </c>
       <c r="E813" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">part of the row's name</t>
+          <t xml:space="preserve">one row per item of the list $.world.factors, in order; a row's name is id, unique</t>
         </is>
       </c>
       <c r="F813" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor's id (the outcomes, leanings and pulls name their factor by it)</t>
+          <t xml:space="preserve">the world's outcomes listed under END OF DEMO, in this order</t>
         </is>
       </c>
     </row>
@@ -20577,7 +20572,7 @@
       </c>
       <c r="B814" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">question</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="C814" s="1" t="inlineStr">
@@ -20587,12 +20582,17 @@
       </c>
       <c r="D814" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">(required)</t>
+        </is>
+      </c>
+      <c r="E814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">part of the row's name</t>
         </is>
       </c>
       <c r="F814" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
+          <t xml:space="preserve">the factor's id (the outcomes, leanings and pulls name their factor by it)</t>
         </is>
       </c>
     </row>
@@ -20604,7 +20604,7 @@
       </c>
       <c r="B815" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">answer</t>
+          <t xml:space="preserve">question</t>
         </is>
       </c>
       <c r="C815" s="1" t="inlineStr">
@@ -20617,14 +20617,9 @@
           <t xml:space="preserve">empty text</t>
         </is>
       </c>
-      <c r="E815" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one of: AsFound, Leader, Pulls</t>
-        </is>
-      </c>
       <c r="F815" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads); Pulls: the outcome the run's choices pull most (worldOutcomes)</t>
+          <t xml:space="preserve">the question the end of the demo answers about 2150</t>
         </is>
       </c>
     </row>
@@ -20636,7 +20631,7 @@
       </c>
       <c r="B816" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">foundAs</t>
+          <t xml:space="preserve">answer</t>
         </is>
       </c>
       <c r="C816" s="1" t="inlineStr">
@@ -20646,12 +20641,17 @@
       </c>
       <c r="D816" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text (left out of the JSON)</t>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E816" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one of: AsFound, Leader, Pulls</t>
         </is>
       </c>
       <c r="F816" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the answer as the run found 2150 (a Pulls factor's is its statusQuo outcome: blank)</t>
+          <t xml:space="preserve">AsFound: the foundAs text; Leader: the leading nation's name (foundAs while none leads); Pulls: the outcome the run's choices pull most (worldOutcomes)</t>
         </is>
       </c>
     </row>
@@ -20663,7 +20663,7 @@
       </c>
       <c r="B817" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">statusQuo</t>
+          <t xml:space="preserve">foundAs</t>
         </is>
       </c>
       <c r="C817" s="1" t="inlineStr">
@@ -20678,7 +20678,7 @@
       </c>
       <c r="F817" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Pulls factor's "as you found it" outcome id: it starts ahead (GameConfigSO worldStatusQuoWeight) and a denial pulls it</t>
+          <t xml:space="preserve">the answer as the run found 2150 (a Pulls factor's is its statusQuo outcome: blank)</t>
         </is>
       </c>
     </row>
@@ -20690,7 +20690,7 @@
       </c>
       <c r="B818" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">splitLine</t>
+          <t xml:space="preserve">statusQuo</t>
         </is>
       </c>
       <c r="C818" s="1" t="inlineStr">
@@ -20705,7 +20705,7 @@
       </c>
       <c r="F818" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Pulls factor's answer when split between two outcomes: {a} and {b} are their names</t>
+          <t xml:space="preserve">a Pulls factor's "as you found it" outcome id: it starts ahead (GameConfigSO worldStatusQuoWeight) and a denial pulls it</t>
         </is>
       </c>
     </row>
@@ -20717,7 +20717,7 @@
       </c>
       <c r="B819" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">splitHeadline</t>
+          <t xml:space="preserve">splitLine</t>
         </is>
       </c>
       <c r="C819" s="1" t="inlineStr">
@@ -20732,29 +20732,34 @@
       </c>
       <c r="F819" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the morning paper's line when the factor splits: {a} and {b}</t>
+          <t xml:space="preserve">a Pulls factor's answer when split between two outcomes: {a} and {b} are their names</t>
         </is>
       </c>
     </row>
     <row r="820">
       <c r="A820" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldOutcomes</t>
+          <t xml:space="preserve">worldFactors</t>
+        </is>
+      </c>
+      <c r="B820" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">splitHeadline</t>
         </is>
       </c>
       <c r="C820" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E820" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.outcomes, in order</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D820" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text (left out of the JSON)</t>
         </is>
       </c>
       <c r="F820" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">every answer of every factor answered by pulls: add rows for more combinations</t>
+          <t xml:space="preserve">the morning paper's line when the factor splits: {a} and {b}</t>
         </is>
       </c>
     </row>
@@ -20764,29 +20769,19 @@
           <t xml:space="preserve">worldOutcomes</t>
         </is>
       </c>
-      <c r="B821" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">factor</t>
-        </is>
-      </c>
       <c r="C821" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D821" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">Rows</t>
         </is>
       </c>
       <c r="E821" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">names a row of 'worldFactors'</t>
+          <t xml:space="preserve">one row per item of the list $.world.outcomes, in order</t>
         </is>
       </c>
       <c r="F821" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor it answers (a Pulls factor)</t>
+          <t xml:space="preserve">every answer of every factor answered by pulls: add rows for more combinations</t>
         </is>
       </c>
     </row>
@@ -20798,7 +20793,7 @@
       </c>
       <c r="B822" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">id</t>
+          <t xml:space="preserve">factor</t>
         </is>
       </c>
       <c r="C822" s="1" t="inlineStr">
@@ -20811,9 +20806,14 @@
           <t xml:space="preserve">(required)</t>
         </is>
       </c>
+      <c r="E822" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'worldFactors'</t>
+        </is>
+      </c>
       <c r="F822" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the outcome's id within its factor (leanings and pulls name it)</t>
+          <t xml:space="preserve">the factor it answers (a Pulls factor)</t>
         </is>
       </c>
     </row>
@@ -20825,7 +20825,7 @@
       </c>
       <c r="B823" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="C823" s="1" t="inlineStr">
@@ -20835,12 +20835,12 @@
       </c>
       <c r="D823" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
+          <t xml:space="preserve">(required)</t>
         </is>
       </c>
       <c r="F823" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the answer as the player reads it</t>
+          <t xml:space="preserve">the outcome's id within its factor (leanings and pulls name it)</t>
         </is>
       </c>
     </row>
@@ -20852,7 +20852,7 @@
       </c>
       <c r="B824" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">headline</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="C824" s="1" t="inlineStr">
@@ -20867,7 +20867,7 @@
       </c>
       <c r="F824" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the morning paper's line the morning after it takes the lead</t>
+          <t xml:space="preserve">the answer as the player reads it</t>
         </is>
       </c>
     </row>
@@ -20879,7 +20879,7 @@
       </c>
       <c r="B825" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">headline</t>
         </is>
       </c>
       <c r="C825" s="1" t="inlineStr">
@@ -20894,29 +20894,34 @@
       </c>
       <c r="F825" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2150 under this answer in a sentence or two, with a joke and an upside, never a verdict</t>
+          <t xml:space="preserve">the morning paper's line the morning after it takes the lead</t>
         </is>
       </c>
     </row>
     <row r="826">
       <c r="A826" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">worldRoles</t>
+          <t xml:space="preserve">worldOutcomes</t>
+        </is>
+      </c>
+      <c r="B826" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
         </is>
       </c>
       <c r="C826" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows</t>
-        </is>
-      </c>
-      <c r="E826" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">one row per item of the list $.world.roles, in order</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D826" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
         </is>
       </c>
       <c r="F826" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">which factor each role pulls; a role not listed pulls nothing</t>
+          <t xml:space="preserve">2150 under this answer in a sentence or two, with a joke and an upside, never a verdict</t>
         </is>
       </c>
     </row>
@@ -20926,24 +20931,19 @@
           <t xml:space="preserve">worldRoles</t>
         </is>
       </c>
-      <c r="B827" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">archetype</t>
-        </is>
-      </c>
       <c r="C827" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="D827" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(required)</t>
+          <t xml:space="preserve">Rows</t>
+        </is>
+      </c>
+      <c r="E827" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one row per item of the list $.world.roles, in order</t>
         </is>
       </c>
       <c r="F827" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">an archetype id (content.archetypes)</t>
+          <t xml:space="preserve">which factor each role pulls; a role not listed pulls nothing</t>
         </is>
       </c>
     </row>
@@ -20955,7 +20955,7 @@
       </c>
       <c r="B828" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">factor</t>
+          <t xml:space="preserve">archetype</t>
         </is>
       </c>
       <c r="C828" s="1" t="inlineStr">
@@ -20965,17 +20965,12 @@
       </c>
       <c r="D828" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">empty text</t>
-        </is>
-      </c>
-      <c r="E828" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">names a row of 'worldFactors'</t>
+          <t xml:space="preserve">(required)</t>
         </is>
       </c>
       <c r="F828" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the factor its accepted travellers pull, toward their destination's leaning</t>
+          <t xml:space="preserve">an archetype id (content.archetypes)</t>
         </is>
       </c>
     </row>
@@ -20987,20 +20982,52 @@
       </c>
       <c r="B829" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">factor</t>
+        </is>
+      </c>
+      <c r="C829" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D829" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty text</t>
+        </is>
+      </c>
+      <c r="E829" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">names a row of 'worldFactors'</t>
+        </is>
+      </c>
+      <c r="F829" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the factor its accepted travellers pull, toward their destination's leaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worldRoles</t>
+        </is>
+      </c>
+      <c r="B830" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">pull</t>
         </is>
       </c>
-      <c r="C829" s="1" t="inlineStr">
+      <c r="C830" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">number</t>
         </is>
       </c>
-      <c r="D829" s="1" t="inlineStr">
+      <c r="D830" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="F829" s="1" t="inlineStr">
+      <c r="F830" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">one accepted traveller's pull, before the kind's scale (GameConfigSO)</t>
         </is>
@@ -24712,16 +24739,17 @@
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
     <col min="3" max="3" width="21" style="1" customWidth="1"/>
-    <col min="4" max="4" width="29" style="1" customWidth="1"/>
-    <col min="5" max="5" width="60" style="1" customWidth="1"/>
-    <col min="6" max="6" width="57" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="1" customWidth="1"/>
-    <col min="9" max="9" width="17" style="1" customWidth="1"/>
-    <col min="10" max="10" width="21" style="1" customWidth="1"/>
-    <col min="11" max="11" width="15" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17" style="1" customWidth="1"/>
-    <col min="13" max="13" width="15" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29" style="1" customWidth="1"/>
+    <col min="6" max="6" width="60" style="1" customWidth="1"/>
+    <col min="7" max="7" width="57" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17" style="1" customWidth="1"/>
+    <col min="11" max="11" width="21" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17" style="1" customWidth="1"/>
+    <col min="14" max="14" width="15" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -24742,50 +24770,55 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">named</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">check</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">against</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">fault</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">point</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">practice.id</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">practice.action</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">practice.categories</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">practice.form</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">practice.target</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">practice.text</t>
         </is>
@@ -24809,20 +24842,25 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Passport</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Its photo and its name.</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">The traveller at the desk: is it their face?</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Someone else's photo: deny.</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">paper:TC-101</t>
         </is>
@@ -24846,20 +24884,25 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">destination</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">The Passport's Destination.</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Today's rule on the RULES tab (from day 3 the Departure Board shows it too).</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Republican Rome on a day only Periclean Athens is open.</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">rulebook</t>
         </is>

</xml_diff>

<commit_message>
feat: stability shown only as the Helix River, never as a number
The desk's stability monitor (the binder lays the river's quad over the
art's StabilityPercent text and switches it off; the art scene untouched),
the PC tray, the shift report ("The timeline tonight") and Home's HUD show
the river; the verdict line, the citation slip and the ledger lose their
stability numbers; the monitor's tooltip names no value. Builders rebuilt
OfficeGameplay and HomeScene; Generate World rebuilt the UI strings; the
firing line and every stability rule are unchanged. Spec:
docs/superpowers/specs/2026-10-07-helix-river-design.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -23066,7 +23066,7 @@
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">الاستقرار: {0}</t>
+          <t xml:space="preserve">الاستقرار</t>
         </is>
       </c>
     </row>
@@ -23576,7 +23576,7 @@
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σταθερότητα: {0}</t>
+          <t xml:space="preserve">Σταθερότητα</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
build: rebuild OfficeGameplay and HomeScene on the integrated head; the pull tabs' word in the card ink
- Build Office UI, Build Home UI and Build Title UI each ran twice:
  idempotent by semantic dump; TitleScene is unchanged; the art scenes are
  byte-unchanged. OfficeGameplay carries every track's builder (the
  daters' lip, the city view's desk controls, the case board, the
  Citation, the memo); HomeScene gains J's serialized pull on SL's machine.
- The readability check failed on the left pull tabs (CITY, PC: 4.36:1, bone
  ink over the tab's sheen, where P's grip-clear word now sits): their word
  is in the palette's card ink (#FAF2E1).
- Generate World ran twice with no change and the validator reports no
  problem; the content template is rewritten for P's sheet map change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ContentSheets/TimeDesk_Content_Template.xlsx
+++ b/ContentSheets/TimeDesk_Content_Template.xlsx
@@ -20029,7 +20029,7 @@
       </c>
       <c r="F791" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">the night's optional bills: the Heating and the TV work only with the Electricity paid</t>
+          <t xml:space="preserve">the night's optional bills: the TV works only with the Electricity paid; the Heating stands alone</t>
         </is>
       </c>
     </row>
@@ -28288,7 +28288,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Click the AVAILABLE sign to call the first traveller.</t>
+          <t xml:space="preserve">Click the AVAILABLE sign to open the desk: the shift clock starts and the first traveller comes.</t>
         </is>
       </c>
     </row>

</xml_diff>